<commit_message>
🚀 [Auto] Sincronização de dados e código
</commit_message>
<xml_diff>
--- a/orcamentos.xlsx
+++ b/orcamentos.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W62"/>
+  <dimension ref="A1:X62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -472,75 +472,80 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
+          <t>currencySymbol</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>status</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>expiredAt</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>refusedAt</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>canceledAt</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>approvedBy</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>createdBy</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>approvedSignature</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>createdAt</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>order.id</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>discount.type</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>discount.value</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>discount.total</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>customer.id</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>location.id</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>status_original</t>
         </is>
@@ -612,61 +617,62 @@
           <t>4000</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
         <is>
           <t>Expirada</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>2025-11-18T15:58:38.481Z</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr">
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr">
         <is>
           <t>Adriana Vieira Masini</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr">
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr">
         <is>
           <t>2025-11-11T16:06:07.949Z</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="R2" t="inlineStr">
         <is>
           <t>NTYyNjA5ODctODA0MS00ODJlLWE1MTQtOTY0ZTQyZWRjOTYwOjU3MDE2</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="S2" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
+      <c r="T2" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr">
+      <c r="U2" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
+      <c r="V2" t="inlineStr">
         <is>
           <t>NDgyMzQxODo1NzAxNg==</t>
         </is>
       </c>
-      <c r="V2" t="inlineStr">
+      <c r="W2" t="inlineStr">
         <is>
           <t>NmFiMDUyZTMtMmRkMi00NWYwLWI1YzAtNzI5N2NmMGJiMzZhOjU3MDE2</t>
         </is>
       </c>
-      <c r="W2" t="inlineStr">
+      <c r="X2" t="inlineStr">
         <is>
           <t>expired</t>
         </is>
@@ -703,69 +709,70 @@
           <t>964.85</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr">
         <is>
           <t>Aprovada</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>2025-11-18T15:45:15.510Z</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr">
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr">
         <is>
           <t>Edina K O Mishima</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>Adriana Vieira Masini</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>accounts/57016/quotations/1774f003-3175-4be8-801c-c7e958af19a8/signatures/650d7c22-e91c-4757-9ac9-9ad5beab0def.png</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="Q3" t="inlineStr">
         <is>
           <t>2025-11-11T15:48:38.327Z</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr">
+      <c r="R3" t="inlineStr">
         <is>
           <t>OTRkZmU3YjYtNDc4OC00OWJlLTk2OWMtYmQ5Y2Q4ZWRiMTY3OjU3MDE2</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr">
+      <c r="S3" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
+      <c r="T3" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr">
+      <c r="U3" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr">
+      <c r="V3" t="inlineStr">
         <is>
           <t>NDgzNDgwNzo1NzAxNg==</t>
         </is>
       </c>
-      <c r="V3" t="inlineStr">
+      <c r="W3" t="inlineStr">
         <is>
           <t>NGNlYTU1YmYtMjg4My00OWI2LWE5YjEtNGEzNTNmZWU3MzZhOjU3MDE2</t>
         </is>
       </c>
-      <c r="W3" t="inlineStr">
+      <c r="X3" t="inlineStr">
         <is>
           <t>approved</t>
         </is>
@@ -806,61 +813,62 @@
           <t>1056.4</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr">
         <is>
           <t>Expirada</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>2025-11-12T12:52:46.887Z</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr">
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr">
         <is>
           <t>Adriana Vieira Masini</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr">
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr">
         <is>
           <t>2025-11-05T13:06:35.085Z</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr">
+      <c r="R4" t="inlineStr">
         <is>
           <t>ZWMwNWE3NTgtODkyOC00ZjE5LWI0YTgtYjY0NmYwMDY2OGIwOjU3MDE2</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
+      <c r="S4" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
+      <c r="T4" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="T4" t="inlineStr">
+      <c r="U4" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr">
+      <c r="V4" t="inlineStr">
         <is>
           <t>NDE2MTc1Nzo1NzAxNg==</t>
         </is>
       </c>
-      <c r="V4" t="inlineStr">
+      <c r="W4" t="inlineStr">
         <is>
           <t>ZDg5NzUyMzktNDc5NS00NDU2LTg0MmItMjZhZjE2MWI3MWUzOjU3MDE2</t>
         </is>
       </c>
-      <c r="W4" t="inlineStr">
+      <c r="X4" t="inlineStr">
         <is>
           <t>expired</t>
         </is>
@@ -897,61 +905,62 @@
           <t>660.525</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr">
         <is>
           <t>Expirada</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>2025-12-18T21:29:48.068Z</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr">
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr">
         <is>
           <t>Adriana Vieira Masini</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr">
+      <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr">
         <is>
           <t>2025-12-11T21:29:54.203Z</t>
         </is>
       </c>
-      <c r="Q5" t="inlineStr">
+      <c r="R5" t="inlineStr">
         <is>
           <t>ZjA3NDk4MWMtM2JiMy00YjVkLTliNTgtYjE3ODFjNjczYmQzOjU3MDE2</t>
         </is>
       </c>
-      <c r="R5" t="inlineStr">
+      <c r="S5" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="S5" t="inlineStr">
+      <c r="T5" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="T5" t="inlineStr">
+      <c r="U5" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U5" t="inlineStr">
+      <c r="V5" t="inlineStr">
         <is>
           <t>NDE3MTYzNjo1NzAxNg==</t>
         </is>
       </c>
-      <c r="V5" t="inlineStr">
+      <c r="W5" t="inlineStr">
         <is>
           <t>ZjZiNTJjY2UtNDFhMS00NjllLTkyNDEtMjIzYmY5ODE2NmJmOjU3MDE2</t>
         </is>
       </c>
-      <c r="W5" t="inlineStr">
+      <c r="X5" t="inlineStr">
         <is>
           <t>expired</t>
         </is>
@@ -992,57 +1001,58 @@
           <t>850.76</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr">
         <is>
           <t>Expirada</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>2026-02-06T18:45:20.986Z</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr">
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr">
         <is>
           <t>Adriana Vieira Masini</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr">
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr">
         <is>
           <t>2026-01-30T18:45:35.907Z</t>
         </is>
       </c>
-      <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr">
+      <c r="R6" t="inlineStr"/>
+      <c r="S6" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="S6" t="inlineStr">
+      <c r="T6" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="T6" t="inlineStr">
+      <c r="U6" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U6" t="inlineStr">
+      <c r="V6" t="inlineStr">
         <is>
           <t>NDM1ODE3Nzo1NzAxNg==</t>
         </is>
       </c>
-      <c r="V6" t="inlineStr">
+      <c r="W6" t="inlineStr">
         <is>
           <t>ZDBlYTE4ZjgtNTRlNS00YjQ2LWIwZDEtZmM2MDc4ZTFhYjY1OjU3MDE2</t>
         </is>
       </c>
-      <c r="W6" t="inlineStr">
+      <c r="X6" t="inlineStr">
         <is>
           <t>expired</t>
         </is>
@@ -1083,65 +1093,66 @@
           <t>350</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr">
         <is>
           <t>Cancelada</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>2026-01-29T14:37:35.560Z</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>2026-01-22T14:57:37.000Z</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="M7" t="inlineStr">
         <is>
           <t>2026-01-22T14:57:37.000Z</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr">
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr">
         <is>
           <t>Lucas Uenishi Tada</t>
         </is>
       </c>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr">
+      <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr">
         <is>
           <t>2026-01-22T14:40:07.831Z</t>
         </is>
       </c>
-      <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr">
+      <c r="R7" t="inlineStr"/>
+      <c r="S7" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="S7" t="inlineStr">
+      <c r="T7" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="T7" t="inlineStr">
+      <c r="U7" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U7" t="inlineStr">
+      <c r="V7" t="inlineStr">
         <is>
           <t>MzMzMDQ1Mjo1NzAxNg==</t>
         </is>
       </c>
-      <c r="V7" t="inlineStr">
+      <c r="W7" t="inlineStr">
         <is>
           <t>YmEwMmQ1NzItYmIwMi00NTAxLWI4NWYtYmZiODY3NjIwZmRhOjU3MDE2</t>
         </is>
       </c>
-      <c r="W7" t="inlineStr">
+      <c r="X7" t="inlineStr">
         <is>
           <t>canceled</t>
         </is>
@@ -1178,61 +1189,62 @@
           <t>300</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr">
         <is>
           <t>Expirada</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>2024-08-14T17:42:21.925Z</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr">
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr">
         <is>
           <t>IRACILDA LOPES</t>
         </is>
       </c>
-      <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr">
+      <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr">
         <is>
           <t>2024-08-07T17:45:02.123Z</t>
         </is>
       </c>
-      <c r="Q8" t="inlineStr">
+      <c r="R8" t="inlineStr">
         <is>
           <t>ZDM4ZDY1NjMtN2E5Yy00ZDQ3LWFlMDktYzUwYzk4NDQ4NWY1OjU3MDE2</t>
         </is>
       </c>
-      <c r="R8" t="inlineStr">
+      <c r="S8" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="S8" t="inlineStr">
+      <c r="T8" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="T8" t="inlineStr">
+      <c r="U8" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U8" t="inlineStr">
+      <c r="V8" t="inlineStr">
         <is>
           <t>MzMxMDM0OTo1NzAxNg==</t>
         </is>
       </c>
-      <c r="V8" t="inlineStr">
+      <c r="W8" t="inlineStr">
         <is>
           <t>MDIzNDM2N2QtZGJmOS00YjhlLTk2ZjUtZWE2N2NlMGVhYjljOjU3MDE2</t>
         </is>
       </c>
-      <c r="W8" t="inlineStr">
+      <c r="X8" t="inlineStr">
         <is>
           <t>expired</t>
         </is>
@@ -1273,65 +1285,66 @@
           <t>1535</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr">
         <is>
           <t>Aprovada</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>2025-09-04T15:24:13.519Z</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr">
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr">
         <is>
           <t>Rafael Machado Barboza</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr">
+      <c r="O9" t="inlineStr">
         <is>
           <t>Adriana Vieira Masini</t>
         </is>
       </c>
-      <c r="O9" t="inlineStr">
+      <c r="P9" t="inlineStr">
         <is>
           <t>accounts/57016/quotations/2a7e8c69-1223-41d3-967d-474788d2fb01/signatures/51c1ade7-ff37-4ee9-b84d-46ee75381607.png</t>
         </is>
       </c>
-      <c r="P9" t="inlineStr">
+      <c r="Q9" t="inlineStr">
         <is>
           <t>2025-08-28T15:35:41.479Z</t>
         </is>
       </c>
-      <c r="Q9" t="inlineStr"/>
-      <c r="R9" t="inlineStr">
+      <c r="R9" t="inlineStr"/>
+      <c r="S9" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="S9" t="inlineStr">
+      <c r="T9" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="T9" t="inlineStr">
+      <c r="U9" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U9" t="inlineStr">
+      <c r="V9" t="inlineStr">
         <is>
           <t>NDIzOTk2OTo1NzAxNg==</t>
         </is>
       </c>
-      <c r="V9" t="inlineStr">
+      <c r="W9" t="inlineStr">
         <is>
           <t>NWY5N2U0ZjYtNjA5Zi00YTkzLWE2ZmQtNjI2YmFhOTU1Y2UzOjU3MDE2</t>
         </is>
       </c>
-      <c r="W9" t="inlineStr">
+      <c r="X9" t="inlineStr">
         <is>
           <t>approved</t>
         </is>
@@ -1376,61 +1389,62 @@
           <t>988.85</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr">
         <is>
           <t>Expirada</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>2025-12-09T21:20:29.860Z</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr">
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr">
         <is>
           <t>Adriana Vieira Masini</t>
         </is>
       </c>
-      <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr">
+      <c r="P10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr">
         <is>
           <t>2025-12-02T21:20:54.686Z</t>
         </is>
       </c>
-      <c r="Q10" t="inlineStr">
+      <c r="R10" t="inlineStr">
         <is>
           <t>ODZlODFiMWItM2FiOC00YmY2LWJiOTktMTExOWE5YzVjMDBjOjU3MDE2</t>
         </is>
       </c>
-      <c r="R10" t="inlineStr">
+      <c r="S10" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="S10" t="inlineStr">
+      <c r="T10" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="T10" t="inlineStr">
+      <c r="U10" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U10" t="inlineStr">
+      <c r="V10" t="inlineStr">
         <is>
           <t>MzI2OTMyNjo1NzAxNg==</t>
         </is>
       </c>
-      <c r="V10" t="inlineStr">
+      <c r="W10" t="inlineStr">
         <is>
           <t>MWUzYmI1OWItNmZiNC00ODg1LTg0ODktOTlmY2IyZWYxNWIxOjU3MDE2</t>
         </is>
       </c>
-      <c r="W10" t="inlineStr">
+      <c r="X10" t="inlineStr">
         <is>
           <t>expired</t>
         </is>
@@ -1467,61 +1481,62 @@
           <t>530.25</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr">
         <is>
           <t>Expirada</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t>2025-10-09T21:18:04.630Z</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr">
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr">
         <is>
           <t>Adriana Vieira Masini</t>
         </is>
       </c>
-      <c r="O11" t="inlineStr"/>
-      <c r="P11" t="inlineStr">
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr">
         <is>
           <t>2025-10-02T21:19:25.794Z</t>
         </is>
       </c>
-      <c r="Q11" t="inlineStr">
+      <c r="R11" t="inlineStr">
         <is>
           <t>OGUzZjA5OGMtMTdlNy00MDY3LTllYjQtMzhmMWNhZGM4NjNmOjU3MDE2</t>
         </is>
       </c>
-      <c r="R11" t="inlineStr">
+      <c r="S11" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="S11" t="inlineStr">
+      <c r="T11" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="T11" t="inlineStr">
+      <c r="U11" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U11" t="inlineStr">
+      <c r="V11" t="inlineStr">
         <is>
           <t>NDcxNTkzODo1NzAxNg==</t>
         </is>
       </c>
-      <c r="V11" t="inlineStr">
+      <c r="W11" t="inlineStr">
         <is>
           <t>MzQwNDRlN2UtMzgxYi00Nzc5LTk1MGItYTY3ODczZDg4NWM0OjU3MDE2</t>
         </is>
       </c>
-      <c r="W11" t="inlineStr">
+      <c r="X11" t="inlineStr">
         <is>
           <t>expired</t>
         </is>
@@ -1562,57 +1577,58 @@
           <t>850.76</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr">
         <is>
           <t>Expirada</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t>2026-01-27T19:18:07.101Z</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr">
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr">
         <is>
           <t>Lucas Uenishi Tada</t>
         </is>
       </c>
-      <c r="O12" t="inlineStr"/>
-      <c r="P12" t="inlineStr">
+      <c r="P12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr">
         <is>
           <t>2026-01-20T19:19:08.741Z</t>
         </is>
       </c>
-      <c r="Q12" t="inlineStr"/>
-      <c r="R12" t="inlineStr">
+      <c r="R12" t="inlineStr"/>
+      <c r="S12" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="S12" t="inlineStr">
+      <c r="T12" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="T12" t="inlineStr">
+      <c r="U12" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U12" t="inlineStr">
+      <c r="V12" t="inlineStr">
         <is>
           <t>NDM1ODE3Nzo1NzAxNg==</t>
         </is>
       </c>
-      <c r="V12" t="inlineStr">
+      <c r="W12" t="inlineStr">
         <is>
           <t>ZDBlYTE4ZjgtNTRlNS00YjQ2LWIwZDEtZmM2MDc4ZTFhYjY1OjU3MDE2</t>
         </is>
       </c>
-      <c r="W12" t="inlineStr">
+      <c r="X12" t="inlineStr">
         <is>
           <t>expired</t>
         </is>
@@ -1657,69 +1673,70 @@
           <t>2167.29</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr">
         <is>
           <t>Aprovada</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="K13" t="inlineStr">
         <is>
           <t>2025-10-06T13:42:48.402Z</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr">
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr">
         <is>
           <t xml:space="preserve">Joana D’Arc Oliveira </t>
         </is>
       </c>
-      <c r="N13" t="inlineStr">
+      <c r="O13" t="inlineStr">
         <is>
           <t>Adriana Vieira Masini</t>
         </is>
       </c>
-      <c r="O13" t="inlineStr">
+      <c r="P13" t="inlineStr">
         <is>
           <t>accounts/57016/quotations/336279a3-e397-43dd-b3ef-8d0f677e97af/signatures/e23e6b48-ded8-4f36-a055-55d66d4bbb0d.png</t>
         </is>
       </c>
-      <c r="P13" t="inlineStr">
+      <c r="Q13" t="inlineStr">
         <is>
           <t>2025-09-29T15:17:10.234Z</t>
         </is>
       </c>
-      <c r="Q13" t="inlineStr">
+      <c r="R13" t="inlineStr">
         <is>
           <t>YTExMmFkNDktMjYyZi00NWVhLWE0Y2YtMjIyZGY1MDc0MjJhOjU3MDE2</t>
         </is>
       </c>
-      <c r="R13" t="inlineStr">
+      <c r="S13" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="S13" t="inlineStr">
+      <c r="T13" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="T13" t="inlineStr">
+      <c r="U13" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U13" t="inlineStr">
+      <c r="V13" t="inlineStr">
         <is>
           <t>MzM3ODI5ODo1NzAxNg==</t>
         </is>
       </c>
-      <c r="V13" t="inlineStr">
+      <c r="W13" t="inlineStr">
         <is>
           <t>MjU3OWZlNzYtYWVlNC00ODU0LWEyYTUtNDdkMWI2ZGY5ZDlmOjU3MDE2</t>
         </is>
       </c>
-      <c r="W13" t="inlineStr">
+      <c r="X13" t="inlineStr">
         <is>
           <t>approved</t>
         </is>
@@ -1756,61 +1773,62 @@
           <t>979.73</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr">
         <is>
           <t>Expirada</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="K14" t="inlineStr">
         <is>
           <t>2025-10-06T18:41:42.725Z</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr">
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr">
         <is>
           <t>Adriana Vieira Masini</t>
         </is>
       </c>
-      <c r="O14" t="inlineStr"/>
-      <c r="P14" t="inlineStr">
+      <c r="P14" t="inlineStr"/>
+      <c r="Q14" t="inlineStr">
         <is>
           <t>2025-09-29T18:42:56.833Z</t>
         </is>
       </c>
-      <c r="Q14" t="inlineStr">
+      <c r="R14" t="inlineStr">
         <is>
           <t>NzdmMmMwZTItZWIyMy00ODUzLWJiZTgtM2Y3YTgzNGM0YzRmOjU3MDE2</t>
         </is>
       </c>
-      <c r="R14" t="inlineStr">
+      <c r="S14" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="S14" t="inlineStr">
+      <c r="T14" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="T14" t="inlineStr">
+      <c r="U14" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U14" t="inlineStr">
+      <c r="V14" t="inlineStr">
         <is>
           <t>MzU0MDM4MDo1NzAxNg==</t>
         </is>
       </c>
-      <c r="V14" t="inlineStr">
+      <c r="W14" t="inlineStr">
         <is>
           <t>MzNhMjk0ZTUtMzI4MS00YTMwLTg2Y2QtYzM3YTQ0OTAyNzI5OjU3MDE2</t>
         </is>
       </c>
-      <c r="W14" t="inlineStr">
+      <c r="X14" t="inlineStr">
         <is>
           <t>expired</t>
         </is>
@@ -1847,61 +1865,62 @@
           <t>1298.9</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr">
         <is>
           <t>Expirada</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="K15" t="inlineStr">
         <is>
           <t>2025-10-06T18:34:31.188Z</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr"/>
-      <c r="N15" t="inlineStr">
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr">
         <is>
           <t>Adriana Vieira Masini</t>
         </is>
       </c>
-      <c r="O15" t="inlineStr"/>
-      <c r="P15" t="inlineStr">
+      <c r="P15" t="inlineStr"/>
+      <c r="Q15" t="inlineStr">
         <is>
           <t>2025-09-29T18:38:37.635Z</t>
         </is>
       </c>
-      <c r="Q15" t="inlineStr">
+      <c r="R15" t="inlineStr">
         <is>
           <t>NzdmMmMwZTItZWIyMy00ODUzLWJiZTgtM2Y3YTgzNGM0YzRmOjU3MDE2</t>
         </is>
       </c>
-      <c r="R15" t="inlineStr">
+      <c r="S15" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="S15" t="inlineStr">
+      <c r="T15" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="T15" t="inlineStr">
+      <c r="U15" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U15" t="inlineStr">
+      <c r="V15" t="inlineStr">
         <is>
           <t>MzU0MDM4MDo1NzAxNg==</t>
         </is>
       </c>
-      <c r="V15" t="inlineStr">
+      <c r="W15" t="inlineStr">
         <is>
           <t>MzNhMjk0ZTUtMzI4MS00YTMwLTg2Y2QtYzM3YTQ0OTAyNzI5OjU3MDE2</t>
         </is>
       </c>
-      <c r="W15" t="inlineStr">
+      <c r="X15" t="inlineStr">
         <is>
           <t>expired</t>
         </is>
@@ -1938,61 +1957,62 @@
           <t>4984</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr">
         <is>
           <t>Expirada</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="K16" t="inlineStr">
         <is>
           <t>2025-10-15T21:09:42.233Z</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr"/>
-      <c r="N16" t="inlineStr">
+      <c r="N16" t="inlineStr"/>
+      <c r="O16" t="inlineStr">
         <is>
           <t>Adriana Vieira Masini</t>
         </is>
       </c>
-      <c r="O16" t="inlineStr"/>
-      <c r="P16" t="inlineStr">
+      <c r="P16" t="inlineStr"/>
+      <c r="Q16" t="inlineStr">
         <is>
           <t>2025-10-08T21:12:33.362Z</t>
         </is>
       </c>
-      <c r="Q16" t="inlineStr">
+      <c r="R16" t="inlineStr">
         <is>
           <t>OTUxMWZiNzEtYjliOC00NTg4LWE5MTAtZmI2ZmQxZmZlZmNlOjU3MDE2</t>
         </is>
       </c>
-      <c r="R16" t="inlineStr">
+      <c r="S16" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="S16" t="inlineStr">
+      <c r="T16" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="T16" t="inlineStr">
+      <c r="U16" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U16" t="inlineStr">
+      <c r="V16" t="inlineStr">
         <is>
           <t>NDgzNDc2OTo1NzAxNg==</t>
         </is>
       </c>
-      <c r="V16" t="inlineStr">
+      <c r="W16" t="inlineStr">
         <is>
           <t>ZThkYWNiNmItMDliOS00Y2Y0LTgyNjgtOGU5OTk4NzQ3MmNkOjU3MDE2</t>
         </is>
       </c>
-      <c r="W16" t="inlineStr">
+      <c r="X16" t="inlineStr">
         <is>
           <t>expired</t>
         </is>
@@ -2034,61 +2054,62 @@
           <t>1016.75</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr">
         <is>
           <t>Expirada</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr">
+      <c r="K17" t="inlineStr">
         <is>
           <t>2025-12-19T15:56:33.655Z</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr"/>
-      <c r="N17" t="inlineStr">
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="inlineStr">
         <is>
           <t>Adriana Vieira Masini</t>
         </is>
       </c>
-      <c r="O17" t="inlineStr"/>
-      <c r="P17" t="inlineStr">
+      <c r="P17" t="inlineStr"/>
+      <c r="Q17" t="inlineStr">
         <is>
           <t>2025-12-12T16:00:42.963Z</t>
         </is>
       </c>
-      <c r="Q17" t="inlineStr">
+      <c r="R17" t="inlineStr">
         <is>
           <t>OTYwNmY5MTktMmQxYi00NzI2LTg3MTYtZTJmMGE1MjE2NjFiOjU3MDE2</t>
         </is>
       </c>
-      <c r="R17" t="inlineStr">
+      <c r="S17" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="S17" t="inlineStr">
+      <c r="T17" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="T17" t="inlineStr">
+      <c r="U17" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U17" t="inlineStr">
+      <c r="V17" t="inlineStr">
         <is>
           <t>MzMxMDI2Nzo1NzAxNg==</t>
         </is>
       </c>
-      <c r="V17" t="inlineStr">
+      <c r="W17" t="inlineStr">
         <is>
           <t>ZWFiZTI5NDgtMzY0Ny00ODVkLThmNjEtODhjMGI2N2Q4Nzk2OjU3MDE2</t>
         </is>
       </c>
-      <c r="W17" t="inlineStr">
+      <c r="X17" t="inlineStr">
         <is>
           <t>expired</t>
         </is>
@@ -2131,61 +2152,62 @@
           <t>350</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr">
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr">
         <is>
           <t>Expirada</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr">
+      <c r="K18" t="inlineStr">
         <is>
           <t>2025-12-24T21:32:57.350Z</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="inlineStr"/>
-      <c r="N18" t="inlineStr">
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="inlineStr">
         <is>
           <t>Adriana Vieira Masini</t>
         </is>
       </c>
-      <c r="O18" t="inlineStr"/>
-      <c r="P18" t="inlineStr">
+      <c r="P18" t="inlineStr"/>
+      <c r="Q18" t="inlineStr">
         <is>
           <t>2025-12-17T21:33:20.182Z</t>
         </is>
       </c>
-      <c r="Q18" t="inlineStr">
+      <c r="R18" t="inlineStr">
         <is>
           <t>ODAxNDQ5MTMtNDYwMi00MjhmLWE1MWUtMWY1Y2I5NGIxY2Y1OjU3MDE2</t>
         </is>
       </c>
-      <c r="R18" t="inlineStr">
+      <c r="S18" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="S18" t="inlineStr">
+      <c r="T18" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="T18" t="inlineStr">
+      <c r="U18" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U18" t="inlineStr">
+      <c r="V18" t="inlineStr">
         <is>
           <t>MzMzMDQ1Mjo1NzAxNg==</t>
         </is>
       </c>
-      <c r="V18" t="inlineStr">
+      <c r="W18" t="inlineStr">
         <is>
           <t>ZTU1NzI4MzEtZTkzNS00ZWIzLTk4MTktMGE3MTZhOTE1NDZlOjU3MDE2</t>
         </is>
       </c>
-      <c r="W18" t="inlineStr">
+      <c r="X18" t="inlineStr">
         <is>
           <t>expired</t>
         </is>
@@ -2222,61 +2244,62 @@
           <t>660.525</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr">
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr">
         <is>
           <t>Expirada</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
+      <c r="K19" t="inlineStr">
         <is>
           <t>2025-11-14T16:10:10.258Z</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr"/>
-      <c r="N19" t="inlineStr">
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr">
         <is>
           <t>Adriana Vieira Masini</t>
         </is>
       </c>
-      <c r="O19" t="inlineStr"/>
-      <c r="P19" t="inlineStr">
+      <c r="P19" t="inlineStr"/>
+      <c r="Q19" t="inlineStr">
         <is>
           <t>2025-11-07T16:26:09.914Z</t>
         </is>
       </c>
-      <c r="Q19" t="inlineStr">
+      <c r="R19" t="inlineStr">
         <is>
           <t>ZjA3NDk4MWMtM2JiMy00YjVkLTliNTgtYjE3ODFjNjczYmQzOjU3MDE2</t>
         </is>
       </c>
-      <c r="R19" t="inlineStr">
+      <c r="S19" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="S19" t="inlineStr">
+      <c r="T19" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="T19" t="inlineStr">
+      <c r="U19" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U19" t="inlineStr">
+      <c r="V19" t="inlineStr">
         <is>
           <t>NDE3MTYzNjo1NzAxNg==</t>
         </is>
       </c>
-      <c r="V19" t="inlineStr">
+      <c r="W19" t="inlineStr">
         <is>
           <t>ZjZiNTJjY2UtNDFhMS00NjllLTkyNDEtMjIzYmY5ODE2NmJmOjU3MDE2</t>
         </is>
       </c>
-      <c r="W19" t="inlineStr">
+      <c r="X19" t="inlineStr">
         <is>
           <t>expired</t>
         </is>
@@ -2317,61 +2340,62 @@
           <t>138.57999999999998</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr">
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr">
         <is>
           <t>Expirada</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr">
+      <c r="K20" t="inlineStr">
         <is>
           <t>2025-12-15T20:05:35.735Z</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr">
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr">
         <is>
           <t>Adriana Vieira Masini</t>
         </is>
       </c>
-      <c r="O20" t="inlineStr"/>
-      <c r="P20" t="inlineStr">
+      <c r="P20" t="inlineStr"/>
+      <c r="Q20" t="inlineStr">
         <is>
           <t>2025-12-08T20:11:36.676Z</t>
         </is>
       </c>
-      <c r="Q20" t="inlineStr">
+      <c r="R20" t="inlineStr">
         <is>
           <t>M2EzOTI5YTItODc3Zi00NTJlLTk1NDktMmU5YWRiMWMwZmQ1OjU3MDE2</t>
         </is>
       </c>
-      <c r="R20" t="inlineStr">
+      <c r="S20" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="S20" t="inlineStr">
+      <c r="T20" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="T20" t="inlineStr">
+      <c r="U20" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U20" t="inlineStr">
+      <c r="V20" t="inlineStr">
         <is>
           <t>NDgzNTU4Mzo1NzAxNg==</t>
         </is>
       </c>
-      <c r="V20" t="inlineStr">
+      <c r="W20" t="inlineStr">
         <is>
           <t>NTk1Y2ZkMTYtMTk4YS00OTE4LWI5YzMtZjcwMTliOTdlNDVjOjU3MDE2</t>
         </is>
       </c>
-      <c r="W20" t="inlineStr">
+      <c r="X20" t="inlineStr">
         <is>
           <t>expired</t>
         </is>
@@ -2416,61 +2440,62 @@
           <t>530.25</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr">
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr">
         <is>
           <t>Expirada</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr">
+      <c r="K21" t="inlineStr">
         <is>
           <t>2025-10-17T12:48:39.389Z</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="inlineStr"/>
-      <c r="N21" t="inlineStr">
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr">
         <is>
           <t>Adriana Vieira Masini</t>
         </is>
       </c>
-      <c r="O21" t="inlineStr"/>
-      <c r="P21" t="inlineStr">
+      <c r="P21" t="inlineStr"/>
+      <c r="Q21" t="inlineStr">
         <is>
           <t>2025-10-10T13:07:18.487Z</t>
         </is>
       </c>
-      <c r="Q21" t="inlineStr">
+      <c r="R21" t="inlineStr">
         <is>
           <t>NGNkMDM2YWEtZDRlMy00NjIwLThiOGMtYmVmNGM1MGMyN2ZkOjU3MDE2</t>
         </is>
       </c>
-      <c r="R21" t="inlineStr">
+      <c r="S21" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="S21" t="inlineStr">
+      <c r="T21" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="T21" t="inlineStr">
+      <c r="U21" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U21" t="inlineStr">
+      <c r="V21" t="inlineStr">
         <is>
           <t>NDgyMzMyODo1NzAxNg==</t>
         </is>
       </c>
-      <c r="V21" t="inlineStr">
+      <c r="W21" t="inlineStr">
         <is>
           <t>NTg2M2M0ZTEtMThhNC00Y2YyLWFhNDktYTViMTdhYzE0MmZmOjU3MDE2</t>
         </is>
       </c>
-      <c r="W21" t="inlineStr">
+      <c r="X21" t="inlineStr">
         <is>
           <t>expired</t>
         </is>
@@ -2515,65 +2540,66 @@
           <t>1047.65</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr">
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr">
         <is>
           <t>Recusada</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr">
+      <c r="K22" t="inlineStr">
         <is>
           <t>2025-11-24T15:13:20.559Z</t>
         </is>
       </c>
-      <c r="K22" t="inlineStr">
+      <c r="L22" t="inlineStr">
         <is>
           <t>2025-11-24T14:45:19.000Z</t>
         </is>
       </c>
-      <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr"/>
-      <c r="N22" t="inlineStr">
+      <c r="N22" t="inlineStr"/>
+      <c r="O22" t="inlineStr">
         <is>
           <t>Adriana Vieira Masini</t>
         </is>
       </c>
-      <c r="O22" t="inlineStr"/>
-      <c r="P22" t="inlineStr">
+      <c r="P22" t="inlineStr"/>
+      <c r="Q22" t="inlineStr">
         <is>
           <t>2025-11-17T15:14:20.735Z</t>
         </is>
       </c>
-      <c r="Q22" t="inlineStr">
+      <c r="R22" t="inlineStr">
         <is>
           <t>ODZlODFiMWItM2FiOC00YmY2LWJiOTktMTExOWE5YzVjMDBjOjU3MDE2</t>
         </is>
       </c>
-      <c r="R22" t="inlineStr">
+      <c r="S22" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="S22" t="inlineStr">
+      <c r="T22" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="T22" t="inlineStr">
+      <c r="U22" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U22" t="inlineStr">
+      <c r="V22" t="inlineStr">
         <is>
           <t>MzI2OTMyNjo1NzAxNg==</t>
         </is>
       </c>
-      <c r="V22" t="inlineStr">
+      <c r="W22" t="inlineStr">
         <is>
           <t>MWUzYmI1OWItNmZiNC00ODg1LTg0ODktOTlmY2IyZWYxNWIxOjU3MDE2</t>
         </is>
       </c>
-      <c r="W22" t="inlineStr">
+      <c r="X22" t="inlineStr">
         <is>
           <t>refused</t>
         </is>
@@ -2615,61 +2641,62 @@
           <t>3000</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr">
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr">
         <is>
           <t>Expirada</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr">
+      <c r="K23" t="inlineStr">
         <is>
           <t>2025-11-25T21:47:25.554Z</t>
         </is>
       </c>
-      <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="inlineStr"/>
-      <c r="N23" t="inlineStr">
+      <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr">
         <is>
           <t>Adriana Vieira Masini</t>
         </is>
       </c>
-      <c r="O23" t="inlineStr"/>
-      <c r="P23" t="inlineStr">
+      <c r="P23" t="inlineStr"/>
+      <c r="Q23" t="inlineStr">
         <is>
           <t>2025-11-18T21:53:35.934Z</t>
         </is>
       </c>
-      <c r="Q23" t="inlineStr">
+      <c r="R23" t="inlineStr">
         <is>
           <t>NjYwZjY1NTAtNjFmZS00N2NmLTlmZTktMzY2ZWVjNmViZGJmOjU3MDE2</t>
         </is>
       </c>
-      <c r="R23" t="inlineStr">
+      <c r="S23" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="S23" t="inlineStr">
+      <c r="T23" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="T23" t="inlineStr">
+      <c r="U23" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U23" t="inlineStr">
+      <c r="V23" t="inlineStr">
         <is>
           <t>NTgwMDkyOTo1NzAxNg==</t>
         </is>
       </c>
-      <c r="V23" t="inlineStr">
+      <c r="W23" t="inlineStr">
         <is>
           <t>YTg3MTBjZDAtMzUwOC00OWNmLWIwMTAtMzMwNGVkOTA5ZWI0OjU3MDE2</t>
         </is>
       </c>
-      <c r="W23" t="inlineStr">
+      <c r="X23" t="inlineStr">
         <is>
           <t>expired</t>
         </is>
@@ -2722,57 +2749,58 @@
           <t>1700</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr">
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr">
         <is>
           <t>Expirada</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr">
+      <c r="K24" t="inlineStr">
         <is>
           <t>2025-09-09T14:06:34.278Z</t>
         </is>
       </c>
-      <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="inlineStr"/>
-      <c r="N24" t="inlineStr">
+      <c r="N24" t="inlineStr"/>
+      <c r="O24" t="inlineStr">
         <is>
           <t>Adriana Vieira Masini</t>
         </is>
       </c>
-      <c r="O24" t="inlineStr"/>
-      <c r="P24" t="inlineStr">
+      <c r="P24" t="inlineStr"/>
+      <c r="Q24" t="inlineStr">
         <is>
           <t>2025-09-02T14:09:17.339Z</t>
         </is>
       </c>
-      <c r="Q24" t="inlineStr"/>
-      <c r="R24" t="inlineStr">
+      <c r="R24" t="inlineStr"/>
+      <c r="S24" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="S24" t="inlineStr">
+      <c r="T24" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="T24" t="inlineStr">
+      <c r="U24" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U24" t="inlineStr">
+      <c r="V24" t="inlineStr">
         <is>
           <t>NDgyMzQxNzo1NzAxNg==</t>
         </is>
       </c>
-      <c r="V24" t="inlineStr">
+      <c r="W24" t="inlineStr">
         <is>
           <t>NTU4NTRiMjItMTA0Yi00ZDEzLThiMDktNzdjYzcxMTFmNzU5OjU3MDE2</t>
         </is>
       </c>
-      <c r="W24" t="inlineStr">
+      <c r="X24" t="inlineStr">
         <is>
           <t>expired</t>
         </is>
@@ -2817,57 +2845,58 @@
           <t>47370</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr">
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr">
         <is>
           <t>Expirada</t>
         </is>
       </c>
-      <c r="J25" t="inlineStr">
+      <c r="K25" t="inlineStr">
         <is>
           <t>2025-08-15T18:25:59.379Z</t>
         </is>
       </c>
-      <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="inlineStr"/>
-      <c r="N25" t="inlineStr">
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr">
         <is>
           <t>RAFAEL BARBOZA</t>
         </is>
       </c>
-      <c r="O25" t="inlineStr"/>
-      <c r="P25" t="inlineStr">
+      <c r="P25" t="inlineStr"/>
+      <c r="Q25" t="inlineStr">
         <is>
           <t>2025-08-08T18:27:17.728Z</t>
         </is>
       </c>
-      <c r="Q25" t="inlineStr"/>
-      <c r="R25" t="inlineStr">
+      <c r="R25" t="inlineStr"/>
+      <c r="S25" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="S25" t="inlineStr">
+      <c r="T25" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="T25" t="inlineStr">
+      <c r="U25" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U25" t="inlineStr">
+      <c r="V25" t="inlineStr">
         <is>
           <t>NDgzNTE2OTo1NzAxNg==</t>
         </is>
       </c>
-      <c r="V25" t="inlineStr">
+      <c r="W25" t="inlineStr">
         <is>
           <t>NzE0ZTQzMTctOWNiOC00OTI2LTgyOTItOWY5NzYxZDE3OGQxOjU3MDE2</t>
         </is>
       </c>
-      <c r="W25" t="inlineStr">
+      <c r="X25" t="inlineStr">
         <is>
           <t>expired</t>
         </is>
@@ -2913,61 +2942,62 @@
           <t>3000</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr">
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr">
         <is>
           <t>Expirada</t>
         </is>
       </c>
-      <c r="J26" t="inlineStr">
+      <c r="K26" t="inlineStr">
         <is>
           <t>2025-12-16T20:19:12.508Z</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="inlineStr"/>
-      <c r="N26" t="inlineStr">
+      <c r="N26" t="inlineStr"/>
+      <c r="O26" t="inlineStr">
         <is>
           <t>Adriana Vieira Masini</t>
         </is>
       </c>
-      <c r="O26" t="inlineStr"/>
-      <c r="P26" t="inlineStr">
+      <c r="P26" t="inlineStr"/>
+      <c r="Q26" t="inlineStr">
         <is>
           <t>2025-12-09T20:21:45.714Z</t>
         </is>
       </c>
-      <c r="Q26" t="inlineStr">
+      <c r="R26" t="inlineStr">
         <is>
           <t>MzIyOGRmMDAtMThlNi00NTc3LTk2MzctYmVjM2QxYmZlOWYwOjU3MDE2</t>
         </is>
       </c>
-      <c r="R26" t="inlineStr">
+      <c r="S26" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="S26" t="inlineStr">
+      <c r="T26" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="T26" t="inlineStr">
+      <c r="U26" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U26" t="inlineStr">
+      <c r="V26" t="inlineStr">
         <is>
           <t>NTg1NDM3Nzo1NzAxNg==</t>
         </is>
       </c>
-      <c r="V26" t="inlineStr">
+      <c r="W26" t="inlineStr">
         <is>
           <t>M2NhMmM5M2MtNWIwNi00OWQwLWFmODgtYTQzNmJiOTUyM2EzOjU3MDE2</t>
         </is>
       </c>
-      <c r="W26" t="inlineStr">
+      <c r="X26" t="inlineStr">
         <is>
           <t>expired</t>
         </is>
@@ -3008,65 +3038,66 @@
           <t>484</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr">
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr">
         <is>
           <t>Aprovada</t>
         </is>
       </c>
-      <c r="J27" t="inlineStr">
+      <c r="K27" t="inlineStr">
         <is>
           <t>2025-12-08T12:21:25.404Z</t>
         </is>
       </c>
-      <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr"/>
-      <c r="M27" t="inlineStr">
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="inlineStr">
         <is>
           <t>douglas simao</t>
         </is>
       </c>
-      <c r="N27" t="inlineStr">
+      <c r="O27" t="inlineStr">
         <is>
           <t>Kaue Teixeira Caldeira Venâncio</t>
         </is>
       </c>
-      <c r="O27" t="inlineStr">
+      <c r="P27" t="inlineStr">
         <is>
           <t>accounts/57016/quotations/6b2b07ff-cb70-450b-bc03-538da26b5fb0/signatures/82045e1d-cc6f-45af-a3f3-2c6a0906455d.png</t>
         </is>
       </c>
-      <c r="P27" t="inlineStr">
+      <c r="Q27" t="inlineStr">
         <is>
           <t>2025-12-01T12:28:02.404Z</t>
         </is>
       </c>
-      <c r="Q27" t="inlineStr"/>
-      <c r="R27" t="inlineStr">
+      <c r="R27" t="inlineStr"/>
+      <c r="S27" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="S27" t="inlineStr">
+      <c r="T27" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="T27" t="inlineStr">
+      <c r="U27" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U27" t="inlineStr">
+      <c r="V27" t="inlineStr">
         <is>
           <t>NDUwNzM2Mzo1NzAxNg==</t>
         </is>
       </c>
-      <c r="V27" t="inlineStr">
+      <c r="W27" t="inlineStr">
         <is>
           <t>ZjBjMzdjOTgtNWY3Yi00ZGQ5LTgwNTktMDZkMjI4YTAzYTAwOjU3MDE2</t>
         </is>
       </c>
-      <c r="W27" t="inlineStr">
+      <c r="X27" t="inlineStr">
         <is>
           <t>approved</t>
         </is>
@@ -3107,61 +3138,62 @@
           <t>5996.77</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr">
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr">
         <is>
           <t>Expirada</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr">
+      <c r="K28" t="inlineStr">
         <is>
           <t>2025-09-15T22:01:12.237Z</t>
         </is>
       </c>
-      <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="inlineStr"/>
-      <c r="N28" t="inlineStr">
+      <c r="N28" t="inlineStr"/>
+      <c r="O28" t="inlineStr">
         <is>
           <t>Adriana Vieira Masini</t>
         </is>
       </c>
-      <c r="O28" t="inlineStr"/>
-      <c r="P28" t="inlineStr">
+      <c r="P28" t="inlineStr"/>
+      <c r="Q28" t="inlineStr">
         <is>
           <t>2025-09-08T22:01:45.251Z</t>
         </is>
       </c>
-      <c r="Q28" t="inlineStr">
+      <c r="R28" t="inlineStr">
         <is>
           <t>ODA0YmUwYWMtMjQ5Ny00MGM4LTgxY2ItYzE2NjBhYzk4MmQxOjU3MDE2</t>
         </is>
       </c>
-      <c r="R28" t="inlineStr">
+      <c r="S28" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="S28" t="inlineStr">
+      <c r="T28" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="T28" t="inlineStr">
+      <c r="U28" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U28" t="inlineStr">
+      <c r="V28" t="inlineStr">
         <is>
           <t>NDIwNTU3Mjo1NzAxNg==</t>
         </is>
       </c>
-      <c r="V28" t="inlineStr">
+      <c r="W28" t="inlineStr">
         <is>
           <t>OTNhMDBkOGItMzEyYy00MzVkLTlmYzItY2I4NWU2ZTQ5MzU5OjU3MDE2</t>
         </is>
       </c>
-      <c r="W28" t="inlineStr">
+      <c r="X28" t="inlineStr">
         <is>
           <t>expired</t>
         </is>
@@ -3202,61 +3234,62 @@
           <t>1756.6</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr">
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr">
         <is>
           <t>Expirada</t>
         </is>
       </c>
-      <c r="J29" t="inlineStr">
+      <c r="K29" t="inlineStr">
         <is>
           <t>2025-12-11T14:05:43.837Z</t>
         </is>
       </c>
-      <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="inlineStr"/>
-      <c r="N29" t="inlineStr">
+      <c r="N29" t="inlineStr"/>
+      <c r="O29" t="inlineStr">
         <is>
           <t>Adriana Vieira Masini</t>
         </is>
       </c>
-      <c r="O29" t="inlineStr"/>
-      <c r="P29" t="inlineStr">
+      <c r="P29" t="inlineStr"/>
+      <c r="Q29" t="inlineStr">
         <is>
           <t>2025-12-04T15:21:12.082Z</t>
         </is>
       </c>
-      <c r="Q29" t="inlineStr">
+      <c r="R29" t="inlineStr">
         <is>
           <t>Y2NjZDRjMTgtOWYwOC00YjUwLWFiNzktOGU0NGNhZTQzMTg3OjU3MDE2</t>
         </is>
       </c>
-      <c r="R29" t="inlineStr">
+      <c r="S29" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="S29" t="inlineStr">
+      <c r="T29" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="T29" t="inlineStr">
+      <c r="U29" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U29" t="inlineStr">
+      <c r="V29" t="inlineStr">
         <is>
           <t>MzUzMTEwNTo1NzAxNg==</t>
         </is>
       </c>
-      <c r="V29" t="inlineStr">
+      <c r="W29" t="inlineStr">
         <is>
           <t>NTM2Nzc5ZjUtZjA3MS00NzY0LTkyNmMtNzQwNmNlZDgzZjEwOjU3MDE2</t>
         </is>
       </c>
-      <c r="W29" t="inlineStr">
+      <c r="X29" t="inlineStr">
         <is>
           <t>expired</t>
         </is>
@@ -3293,61 +3326,62 @@
           <t>490.38</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr">
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr">
         <is>
           <t>Expirada</t>
         </is>
       </c>
-      <c r="J30" t="inlineStr">
+      <c r="K30" t="inlineStr">
         <is>
           <t>2025-10-06T18:43:16.449Z</t>
         </is>
       </c>
-      <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="inlineStr"/>
-      <c r="N30" t="inlineStr">
+      <c r="N30" t="inlineStr"/>
+      <c r="O30" t="inlineStr">
         <is>
           <t>Adriana Vieira Masini</t>
         </is>
       </c>
-      <c r="O30" t="inlineStr"/>
-      <c r="P30" t="inlineStr">
+      <c r="P30" t="inlineStr"/>
+      <c r="Q30" t="inlineStr">
         <is>
           <t>2025-09-29T18:44:47.397Z</t>
         </is>
       </c>
-      <c r="Q30" t="inlineStr">
+      <c r="R30" t="inlineStr">
         <is>
           <t>NzdmMmMwZTItZWIyMy00ODUzLWJiZTgtM2Y3YTgzNGM0YzRmOjU3MDE2</t>
         </is>
       </c>
-      <c r="R30" t="inlineStr">
+      <c r="S30" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="S30" t="inlineStr">
+      <c r="T30" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="T30" t="inlineStr">
+      <c r="U30" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U30" t="inlineStr">
+      <c r="V30" t="inlineStr">
         <is>
           <t>MzU0MDM4MDo1NzAxNg==</t>
         </is>
       </c>
-      <c r="V30" t="inlineStr">
+      <c r="W30" t="inlineStr">
         <is>
           <t>MzNhMjk0ZTUtMzI4MS00YTMwLTg2Y2QtYzM3YTQ0OTAyNzI5OjU3MDE2</t>
         </is>
       </c>
-      <c r="W30" t="inlineStr">
+      <c r="X30" t="inlineStr">
         <is>
           <t>expired</t>
         </is>
@@ -3392,57 +3426,58 @@
           <t>1535</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr">
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr">
         <is>
           <t>Expirada</t>
         </is>
       </c>
-      <c r="J31" t="inlineStr">
+      <c r="K31" t="inlineStr">
         <is>
           <t>2025-09-04T16:01:06.048Z</t>
         </is>
       </c>
-      <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="inlineStr"/>
-      <c r="N31" t="inlineStr">
+      <c r="N31" t="inlineStr"/>
+      <c r="O31" t="inlineStr">
         <is>
           <t>Adriana Vieira Masini</t>
         </is>
       </c>
-      <c r="O31" t="inlineStr"/>
-      <c r="P31" t="inlineStr">
+      <c r="P31" t="inlineStr"/>
+      <c r="Q31" t="inlineStr">
         <is>
           <t>2025-08-28T16:05:56.490Z</t>
         </is>
       </c>
-      <c r="Q31" t="inlineStr"/>
-      <c r="R31" t="inlineStr">
+      <c r="R31" t="inlineStr"/>
+      <c r="S31" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="S31" t="inlineStr">
+      <c r="T31" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="T31" t="inlineStr">
+      <c r="U31" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U31" t="inlineStr">
+      <c r="V31" t="inlineStr">
         <is>
           <t>NDIzOTk2OTo1NzAxNg==</t>
         </is>
       </c>
-      <c r="V31" t="inlineStr">
+      <c r="W31" t="inlineStr">
         <is>
           <t>NWY5N2U0ZjYtNjA5Zi00YTkzLWE2ZmQtNjI2YmFhOTU1Y2UzOjU3MDE2</t>
         </is>
       </c>
-      <c r="W31" t="inlineStr">
+      <c r="X31" t="inlineStr">
         <is>
           <t>expired</t>
         </is>
@@ -3483,57 +3518,58 @@
           <t>660.525</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr">
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr">
         <is>
           <t>Expirada</t>
         </is>
       </c>
-      <c r="J32" t="inlineStr">
+      <c r="K32" t="inlineStr">
         <is>
           <t>2026-01-29T17:13:31.699Z</t>
         </is>
       </c>
-      <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr"/>
       <c r="M32" t="inlineStr"/>
-      <c r="N32" t="inlineStr">
+      <c r="N32" t="inlineStr"/>
+      <c r="O32" t="inlineStr">
         <is>
           <t>Lucas Uenishi Tada</t>
         </is>
       </c>
-      <c r="O32" t="inlineStr"/>
-      <c r="P32" t="inlineStr">
+      <c r="P32" t="inlineStr"/>
+      <c r="Q32" t="inlineStr">
         <is>
           <t>2026-01-22T17:24:06.452Z</t>
         </is>
       </c>
-      <c r="Q32" t="inlineStr"/>
-      <c r="R32" t="inlineStr">
+      <c r="R32" t="inlineStr"/>
+      <c r="S32" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="S32" t="inlineStr">
+      <c r="T32" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="T32" t="inlineStr">
+      <c r="U32" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U32" t="inlineStr">
+      <c r="V32" t="inlineStr">
         <is>
           <t>NDgyNDM2OTo1NzAxNg==</t>
         </is>
       </c>
-      <c r="V32" t="inlineStr">
+      <c r="W32" t="inlineStr">
         <is>
           <t>MTU0OGJhYjItYzE4NS00NGNmLThhOGItYzA1MzhmNTNjODJlOjU3MDE2</t>
         </is>
       </c>
-      <c r="W32" t="inlineStr">
+      <c r="X32" t="inlineStr">
         <is>
           <t>expired</t>
         </is>
@@ -3574,57 +3610,58 @@
           <t>350</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr">
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr">
         <is>
           <t>Expirada</t>
         </is>
       </c>
-      <c r="J33" t="inlineStr">
+      <c r="K33" t="inlineStr">
         <is>
           <t>2026-01-29T12:16:04.953Z</t>
         </is>
       </c>
-      <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr"/>
       <c r="M33" t="inlineStr"/>
-      <c r="N33" t="inlineStr">
+      <c r="N33" t="inlineStr"/>
+      <c r="O33" t="inlineStr">
         <is>
           <t>Lucas Uenishi Tada</t>
         </is>
       </c>
-      <c r="O33" t="inlineStr"/>
-      <c r="P33" t="inlineStr">
+      <c r="P33" t="inlineStr"/>
+      <c r="Q33" t="inlineStr">
         <is>
           <t>2026-01-22T13:01:41.368Z</t>
         </is>
       </c>
-      <c r="Q33" t="inlineStr"/>
-      <c r="R33" t="inlineStr">
+      <c r="R33" t="inlineStr"/>
+      <c r="S33" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="S33" t="inlineStr">
+      <c r="T33" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="T33" t="inlineStr">
+      <c r="U33" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U33" t="inlineStr">
+      <c r="V33" t="inlineStr">
         <is>
           <t>MzMzMDQ1Mjo1NzAxNg==</t>
         </is>
       </c>
-      <c r="V33" t="inlineStr">
+      <c r="W33" t="inlineStr">
         <is>
           <t>YmEwMmQ1NzItYmIwMi00NTAxLWI4NWYtYmZiODY3NjIwZmRhOjU3MDE2</t>
         </is>
       </c>
-      <c r="W33" t="inlineStr">
+      <c r="X33" t="inlineStr">
         <is>
           <t>expired</t>
         </is>
@@ -3665,61 +3702,62 @@
           <t>478</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr">
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr">
         <is>
           <t>Expirada</t>
         </is>
       </c>
-      <c r="J34" t="inlineStr">
+      <c r="K34" t="inlineStr">
         <is>
           <t>2025-11-10T19:48:40.136Z</t>
         </is>
       </c>
-      <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr"/>
       <c r="M34" t="inlineStr"/>
-      <c r="N34" t="inlineStr">
+      <c r="N34" t="inlineStr"/>
+      <c r="O34" t="inlineStr">
         <is>
           <t>Adriana Vieira Masini</t>
         </is>
       </c>
-      <c r="O34" t="inlineStr"/>
-      <c r="P34" t="inlineStr">
+      <c r="P34" t="inlineStr"/>
+      <c r="Q34" t="inlineStr">
         <is>
           <t>2025-11-03T19:49:41.839Z</t>
         </is>
       </c>
-      <c r="Q34" t="inlineStr">
+      <c r="R34" t="inlineStr">
         <is>
           <t>MGIyNGUzMWQtMDM4OS00ZDc1LTg5MGEtYmNiNzViYTNjNGFiOjU3MDE2</t>
         </is>
       </c>
-      <c r="R34" t="inlineStr">
+      <c r="S34" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="S34" t="inlineStr">
+      <c r="T34" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="T34" t="inlineStr">
+      <c r="U34" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U34" t="inlineStr">
+      <c r="V34" t="inlineStr">
         <is>
           <t>NDgyMzkyMzo1NzAxNg==</t>
         </is>
       </c>
-      <c r="V34" t="inlineStr">
+      <c r="W34" t="inlineStr">
         <is>
           <t>MmJlOTE4ZTYtMjdkMy00NThjLWE0ODUtYjczNjgwYjM3NWJhOjU3MDE2</t>
         </is>
       </c>
-      <c r="W34" t="inlineStr">
+      <c r="X34" t="inlineStr">
         <is>
           <t>expired</t>
         </is>
@@ -3760,65 +3798,66 @@
           <t>9000</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr">
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr">
         <is>
           <t>Aprovada</t>
         </is>
       </c>
-      <c r="J35" t="inlineStr">
+      <c r="K35" t="inlineStr">
         <is>
           <t>2023-06-07T21:55:05.692Z</t>
         </is>
       </c>
-      <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr"/>
-      <c r="M35" t="inlineStr">
+      <c r="M35" t="inlineStr"/>
+      <c r="N35" t="inlineStr">
         <is>
           <t>jose da silva</t>
         </is>
       </c>
-      <c r="N35" t="inlineStr">
+      <c r="O35" t="inlineStr">
         <is>
           <t>HENRIQUE</t>
         </is>
       </c>
-      <c r="O35" t="inlineStr">
+      <c r="P35" t="inlineStr">
         <is>
           <t>accounts/57016/quotations/913c656d-9e89-4cee-bb63-5297f22057c5/signatures/a8215aae-2f41-4179-a1ba-a923278bb210.png</t>
         </is>
       </c>
-      <c r="P35" t="inlineStr">
+      <c r="Q35" t="inlineStr">
         <is>
           <t>2023-05-31T21:56:50.448Z</t>
         </is>
       </c>
-      <c r="Q35" t="inlineStr"/>
-      <c r="R35" t="inlineStr">
+      <c r="R35" t="inlineStr"/>
+      <c r="S35" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="S35" t="inlineStr">
+      <c r="T35" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="T35" t="inlineStr">
+      <c r="U35" t="inlineStr">
         <is>
           <t>1000</t>
         </is>
       </c>
-      <c r="U35" t="inlineStr">
+      <c r="V35" t="inlineStr">
         <is>
           <t>MzE2ODMzNTo1NzAxNg==</t>
         </is>
       </c>
-      <c r="V35" t="inlineStr">
+      <c r="W35" t="inlineStr">
         <is>
           <t>YmViOGRmMjAtM2EwYy00NTFkLTkwNzctODkwYmM4MzA5NGQ0OjU3MDE2</t>
         </is>
       </c>
-      <c r="W35" t="inlineStr">
+      <c r="X35" t="inlineStr">
         <is>
           <t>approved</t>
         </is>
@@ -3859,61 +3898,62 @@
           <t>1298.9</t>
         </is>
       </c>
-      <c r="I36" t="inlineStr">
+      <c r="I36" t="inlineStr"/>
+      <c r="J36" t="inlineStr">
         <is>
           <t>Expirada</t>
         </is>
       </c>
-      <c r="J36" t="inlineStr">
+      <c r="K36" t="inlineStr">
         <is>
           <t>2025-11-13T15:27:58.539Z</t>
         </is>
       </c>
-      <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr"/>
       <c r="M36" t="inlineStr"/>
-      <c r="N36" t="inlineStr">
+      <c r="N36" t="inlineStr"/>
+      <c r="O36" t="inlineStr">
         <is>
           <t>Kaue Teixeira Caldeira Venâncio</t>
         </is>
       </c>
-      <c r="O36" t="inlineStr"/>
-      <c r="P36" t="inlineStr">
+      <c r="P36" t="inlineStr"/>
+      <c r="Q36" t="inlineStr">
         <is>
           <t>2025-11-06T15:28:06.348Z</t>
         </is>
       </c>
-      <c r="Q36" t="inlineStr">
+      <c r="R36" t="inlineStr">
         <is>
           <t>NzdmMmMwZTItZWIyMy00ODUzLWJiZTgtM2Y3YTgzNGM0YzRmOjU3MDE2</t>
         </is>
       </c>
-      <c r="R36" t="inlineStr">
+      <c r="S36" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="S36" t="inlineStr">
+      <c r="T36" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="T36" t="inlineStr">
+      <c r="U36" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U36" t="inlineStr">
+      <c r="V36" t="inlineStr">
         <is>
           <t>MzU0MDM4MDo1NzAxNg==</t>
         </is>
       </c>
-      <c r="V36" t="inlineStr">
+      <c r="W36" t="inlineStr">
         <is>
           <t>MzNhMjk0ZTUtMzI4MS00YTMwLTg2Y2QtYzM3YTQ0OTAyNzI5OjU3MDE2</t>
         </is>
       </c>
-      <c r="W36" t="inlineStr">
+      <c r="X36" t="inlineStr">
         <is>
           <t>expired</t>
         </is>
@@ -3954,65 +3994,66 @@
           <t>1535</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr">
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="inlineStr">
         <is>
           <t>Aprovada</t>
         </is>
       </c>
-      <c r="J37" t="inlineStr">
+      <c r="K37" t="inlineStr">
         <is>
           <t>2025-09-04T16:07:52.834Z</t>
         </is>
       </c>
-      <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr"/>
-      <c r="M37" t="inlineStr">
+      <c r="M37" t="inlineStr"/>
+      <c r="N37" t="inlineStr">
         <is>
           <t>rffccfc</t>
         </is>
       </c>
-      <c r="N37" t="inlineStr">
+      <c r="O37" t="inlineStr">
         <is>
           <t>Adriana Vieira Masini</t>
         </is>
       </c>
-      <c r="O37" t="inlineStr">
+      <c r="P37" t="inlineStr">
         <is>
           <t>accounts/57016/quotations/970cf169-2b55-4eed-b7bc-c418d38522f4/signatures/7a22a671-9310-4602-ba1e-f1006682889f.png</t>
         </is>
       </c>
-      <c r="P37" t="inlineStr">
+      <c r="Q37" t="inlineStr">
         <is>
           <t>2025-08-28T16:10:11.398Z</t>
         </is>
       </c>
-      <c r="Q37" t="inlineStr"/>
-      <c r="R37" t="inlineStr">
+      <c r="R37" t="inlineStr"/>
+      <c r="S37" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="S37" t="inlineStr">
+      <c r="T37" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="T37" t="inlineStr">
+      <c r="U37" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U37" t="inlineStr">
+      <c r="V37" t="inlineStr">
         <is>
           <t>NDIzOTk2OTo1NzAxNg==</t>
         </is>
       </c>
-      <c r="V37" t="inlineStr">
+      <c r="W37" t="inlineStr">
         <is>
           <t>NWY5N2U0ZjYtNjA5Zi00YTkzLWE2ZmQtNjI2YmFhOTU1Y2UzOjU3MDE2</t>
         </is>
       </c>
-      <c r="W37" t="inlineStr">
+      <c r="X37" t="inlineStr">
         <is>
           <t>approved</t>
         </is>
@@ -4049,57 +4090,58 @@
           <t>40.894999999999996</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr">
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr">
         <is>
           <t>Expirada</t>
         </is>
       </c>
-      <c r="J38" t="inlineStr">
+      <c r="K38" t="inlineStr">
         <is>
           <t>2025-10-20T12:54:09.917Z</t>
         </is>
       </c>
-      <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr"/>
       <c r="M38" t="inlineStr"/>
-      <c r="N38" t="inlineStr">
+      <c r="N38" t="inlineStr"/>
+      <c r="O38" t="inlineStr">
         <is>
           <t>Kaue Teixeira Caldeira Venâncio</t>
         </is>
       </c>
-      <c r="O38" t="inlineStr"/>
-      <c r="P38" t="inlineStr">
+      <c r="P38" t="inlineStr"/>
+      <c r="Q38" t="inlineStr">
         <is>
           <t>2025-10-13T13:10:02.576Z</t>
         </is>
       </c>
-      <c r="Q38" t="inlineStr"/>
-      <c r="R38" t="inlineStr">
+      <c r="R38" t="inlineStr"/>
+      <c r="S38" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="S38" t="inlineStr">
+      <c r="T38" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="T38" t="inlineStr">
+      <c r="U38" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U38" t="inlineStr">
+      <c r="V38" t="inlineStr">
         <is>
           <t>NDgyNTIyNjo1NzAxNg==</t>
         </is>
       </c>
-      <c r="V38" t="inlineStr">
+      <c r="W38" t="inlineStr">
         <is>
           <t>YTg2MWYxNTktMTEyNi00YWYxLWI4MmMtNzBlODk1NDQwMjE3OjU3MDE2</t>
         </is>
       </c>
-      <c r="W38" t="inlineStr">
+      <c r="X38" t="inlineStr">
         <is>
           <t>expired</t>
         </is>
@@ -4140,61 +4182,62 @@
           <t>47370</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr">
+      <c r="I39" t="inlineStr"/>
+      <c r="J39" t="inlineStr">
         <is>
           <t>Recusada</t>
         </is>
       </c>
-      <c r="J39" t="inlineStr">
+      <c r="K39" t="inlineStr">
         <is>
           <t>2025-08-15T18:20:20.020Z</t>
         </is>
       </c>
-      <c r="K39" t="inlineStr">
+      <c r="L39" t="inlineStr">
         <is>
           <t>2025-08-08T18:24:47.000Z</t>
         </is>
       </c>
-      <c r="L39" t="inlineStr"/>
       <c r="M39" t="inlineStr"/>
-      <c r="N39" t="inlineStr">
+      <c r="N39" t="inlineStr"/>
+      <c r="O39" t="inlineStr">
         <is>
           <t>RAFAEL BARBOZA</t>
         </is>
       </c>
-      <c r="O39" t="inlineStr"/>
-      <c r="P39" t="inlineStr">
+      <c r="P39" t="inlineStr"/>
+      <c r="Q39" t="inlineStr">
         <is>
           <t>2025-08-08T18:23:10.037Z</t>
         </is>
       </c>
-      <c r="Q39" t="inlineStr"/>
-      <c r="R39" t="inlineStr">
+      <c r="R39" t="inlineStr"/>
+      <c r="S39" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="S39" t="inlineStr">
+      <c r="T39" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="T39" t="inlineStr">
+      <c r="U39" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U39" t="inlineStr">
+      <c r="V39" t="inlineStr">
         <is>
           <t>NDgzNTE2OTo1NzAxNg==</t>
         </is>
       </c>
-      <c r="V39" t="inlineStr">
+      <c r="W39" t="inlineStr">
         <is>
           <t>NzE0ZTQzMTctOWNiOC00OTI2LTgyOTItOWY5NzYxZDE3OGQxOjU3MDE2</t>
         </is>
       </c>
-      <c r="W39" t="inlineStr">
+      <c r="X39" t="inlineStr">
         <is>
           <t>refused</t>
         </is>
@@ -4235,61 +4278,62 @@
           <t>451.5</t>
         </is>
       </c>
-      <c r="I40" t="inlineStr">
+      <c r="I40" t="inlineStr"/>
+      <c r="J40" t="inlineStr">
         <is>
           <t>Expirada</t>
         </is>
       </c>
-      <c r="J40" t="inlineStr">
+      <c r="K40" t="inlineStr">
         <is>
           <t>2025-12-19T16:01:13.514Z</t>
         </is>
       </c>
-      <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr"/>
       <c r="M40" t="inlineStr"/>
-      <c r="N40" t="inlineStr">
+      <c r="N40" t="inlineStr"/>
+      <c r="O40" t="inlineStr">
         <is>
           <t>Adriana Vieira Masini</t>
         </is>
       </c>
-      <c r="O40" t="inlineStr"/>
-      <c r="P40" t="inlineStr">
+      <c r="P40" t="inlineStr"/>
+      <c r="Q40" t="inlineStr">
         <is>
           <t>2025-12-12T16:02:27.309Z</t>
         </is>
       </c>
-      <c r="Q40" t="inlineStr">
+      <c r="R40" t="inlineStr">
         <is>
           <t>OTYwNmY5MTktMmQxYi00NzI2LTg3MTYtZTJmMGE1MjE2NjFiOjU3MDE2</t>
         </is>
       </c>
-      <c r="R40" t="inlineStr">
+      <c r="S40" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="S40" t="inlineStr">
+      <c r="T40" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="T40" t="inlineStr">
+      <c r="U40" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U40" t="inlineStr">
+      <c r="V40" t="inlineStr">
         <is>
           <t>MzMxMDI2Nzo1NzAxNg==</t>
         </is>
       </c>
-      <c r="V40" t="inlineStr">
+      <c r="W40" t="inlineStr">
         <is>
           <t>ZWFiZTI5NDgtMzY0Ny00ODVkLThmNjEtODhjMGI2N2Q4Nzk2OjU3MDE2</t>
         </is>
       </c>
-      <c r="W40" t="inlineStr">
+      <c r="X40" t="inlineStr">
         <is>
           <t>expired</t>
         </is>
@@ -4326,61 +4370,62 @@
           <t>0.01</t>
         </is>
       </c>
-      <c r="I41" t="inlineStr">
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" t="inlineStr">
         <is>
           <t>Expirada</t>
         </is>
       </c>
-      <c r="J41" t="inlineStr">
+      <c r="K41" t="inlineStr">
         <is>
           <t>2024-09-12T20:48:10.536Z</t>
         </is>
       </c>
-      <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr"/>
       <c r="M41" t="inlineStr"/>
-      <c r="N41" t="inlineStr">
+      <c r="N41" t="inlineStr"/>
+      <c r="O41" t="inlineStr">
         <is>
           <t>Adriana Vieira Masini</t>
         </is>
       </c>
-      <c r="O41" t="inlineStr"/>
-      <c r="P41" t="inlineStr">
+      <c r="P41" t="inlineStr"/>
+      <c r="Q41" t="inlineStr">
         <is>
           <t>2024-09-05T20:49:15.417Z</t>
         </is>
       </c>
-      <c r="Q41" t="inlineStr">
+      <c r="R41" t="inlineStr">
         <is>
           <t>Zjc2MWE3MWQtNDExOS00NDVmLWFkZmUtNzNlY2M3NmMwNGEyOjU3MDE2</t>
         </is>
       </c>
-      <c r="R41" t="inlineStr">
+      <c r="S41" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="S41" t="inlineStr">
+      <c r="T41" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="T41" t="inlineStr">
+      <c r="U41" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U41" t="inlineStr">
+      <c r="V41" t="inlineStr">
         <is>
           <t>NDIxMTExMTo1NzAxNg==</t>
         </is>
       </c>
-      <c r="V41" t="inlineStr">
+      <c r="W41" t="inlineStr">
         <is>
           <t>ZmU4N2U3MGQtMzJiMi00MDhlLTljNzktZTRmN2M1ZDcyNzUwOjU3MDE2</t>
         </is>
       </c>
-      <c r="W41" t="inlineStr">
+      <c r="X41" t="inlineStr">
         <is>
           <t>expired</t>
         </is>
@@ -4421,57 +4466,58 @@
           <t>3000</t>
         </is>
       </c>
-      <c r="I42" t="inlineStr">
+      <c r="I42" t="inlineStr"/>
+      <c r="J42" t="inlineStr">
         <is>
           <t>Expirada</t>
         </is>
       </c>
-      <c r="J42" t="inlineStr">
+      <c r="K42" t="inlineStr">
         <is>
           <t>2026-01-23T17:25:57.681Z</t>
         </is>
       </c>
-      <c r="K42" t="inlineStr"/>
       <c r="L42" t="inlineStr"/>
       <c r="M42" t="inlineStr"/>
-      <c r="N42" t="inlineStr">
+      <c r="N42" t="inlineStr"/>
+      <c r="O42" t="inlineStr">
         <is>
           <t>Kaue Teixeira Caldeira Venâncio</t>
         </is>
       </c>
-      <c r="O42" t="inlineStr"/>
-      <c r="P42" t="inlineStr">
+      <c r="P42" t="inlineStr"/>
+      <c r="Q42" t="inlineStr">
         <is>
           <t>2026-01-16T17:30:58.730Z</t>
         </is>
       </c>
-      <c r="Q42" t="inlineStr"/>
-      <c r="R42" t="inlineStr">
+      <c r="R42" t="inlineStr"/>
+      <c r="S42" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="S42" t="inlineStr">
+      <c r="T42" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="T42" t="inlineStr">
+      <c r="U42" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U42" t="inlineStr">
+      <c r="V42" t="inlineStr">
         <is>
           <t>NDgyNTk1Mzo1NzAxNg==</t>
         </is>
       </c>
-      <c r="V42" t="inlineStr">
+      <c r="W42" t="inlineStr">
         <is>
           <t>MzMzMDQ3ZTYtMzU1OC00MTZjLWExZGYtNWU4MTg4ZmY2YzdhOjU3MDE2</t>
         </is>
       </c>
-      <c r="W42" t="inlineStr">
+      <c r="X42" t="inlineStr">
         <is>
           <t>expired</t>
         </is>
@@ -4522,61 +4568,62 @@
           <t>1700</t>
         </is>
       </c>
-      <c r="I43" t="inlineStr">
+      <c r="I43" t="inlineStr"/>
+      <c r="J43" t="inlineStr">
         <is>
           <t>Expirada</t>
         </is>
       </c>
-      <c r="J43" t="inlineStr">
+      <c r="K43" t="inlineStr">
         <is>
           <t>2025-09-09T13:53:17.012Z</t>
         </is>
       </c>
-      <c r="K43" t="inlineStr"/>
       <c r="L43" t="inlineStr"/>
       <c r="M43" t="inlineStr"/>
-      <c r="N43" t="inlineStr">
+      <c r="N43" t="inlineStr"/>
+      <c r="O43" t="inlineStr">
         <is>
           <t>Adriana Vieira Masini</t>
         </is>
       </c>
-      <c r="O43" t="inlineStr"/>
-      <c r="P43" t="inlineStr">
+      <c r="P43" t="inlineStr"/>
+      <c r="Q43" t="inlineStr">
         <is>
           <t>2025-09-02T14:01:32.021Z</t>
         </is>
       </c>
-      <c r="Q43" t="inlineStr">
+      <c r="R43" t="inlineStr">
         <is>
           <t>MTk4MjI5MTUtMDk1NC00NWFhLWE0NmEtMWJlMWZkYzdjMGVmOjU3MDE2</t>
         </is>
       </c>
-      <c r="R43" t="inlineStr">
+      <c r="S43" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="S43" t="inlineStr">
+      <c r="T43" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="T43" t="inlineStr">
+      <c r="U43" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U43" t="inlineStr">
+      <c r="V43" t="inlineStr">
         <is>
           <t>NDgyMzQxNzo1NzAxNg==</t>
         </is>
       </c>
-      <c r="V43" t="inlineStr">
+      <c r="W43" t="inlineStr">
         <is>
           <t>NTU4NTRiMjItMTA0Yi00ZDEzLThiMDktNzdjYzcxMTFmNzU5OjU3MDE2</t>
         </is>
       </c>
-      <c r="W43" t="inlineStr">
+      <c r="X43" t="inlineStr">
         <is>
           <t>expired</t>
         </is>
@@ -4617,57 +4664,58 @@
           <t>5996.77</t>
         </is>
       </c>
-      <c r="I44" t="inlineStr">
+      <c r="I44" t="inlineStr"/>
+      <c r="J44" t="inlineStr">
         <is>
           <t>Expirada</t>
         </is>
       </c>
-      <c r="J44" t="inlineStr">
+      <c r="K44" t="inlineStr">
         <is>
           <t>2025-09-15T21:48:09.008Z</t>
         </is>
       </c>
-      <c r="K44" t="inlineStr"/>
       <c r="L44" t="inlineStr"/>
       <c r="M44" t="inlineStr"/>
-      <c r="N44" t="inlineStr">
+      <c r="N44" t="inlineStr"/>
+      <c r="O44" t="inlineStr">
         <is>
           <t>Adriana Vieira Masini</t>
         </is>
       </c>
-      <c r="O44" t="inlineStr"/>
-      <c r="P44" t="inlineStr">
+      <c r="P44" t="inlineStr"/>
+      <c r="Q44" t="inlineStr">
         <is>
           <t>2025-09-08T21:59:15.256Z</t>
         </is>
       </c>
-      <c r="Q44" t="inlineStr"/>
-      <c r="R44" t="inlineStr">
+      <c r="R44" t="inlineStr"/>
+      <c r="S44" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="S44" t="inlineStr">
+      <c r="T44" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="T44" t="inlineStr">
+      <c r="U44" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U44" t="inlineStr">
+      <c r="V44" t="inlineStr">
         <is>
           <t>NDIwNTU3Mjo1NzAxNg==</t>
         </is>
       </c>
-      <c r="V44" t="inlineStr">
+      <c r="W44" t="inlineStr">
         <is>
           <t>OTNhMDBkOGItMzEyYy00MzVkLTlmYzItY2I4NWU2ZTQ5MzU5OjU3MDE2</t>
         </is>
       </c>
-      <c r="W44" t="inlineStr">
+      <c r="X44" t="inlineStr">
         <is>
           <t>expired</t>
         </is>
@@ -4708,61 +4756,62 @@
           <t>490.38</t>
         </is>
       </c>
-      <c r="I45" t="inlineStr">
+      <c r="I45" t="inlineStr"/>
+      <c r="J45" t="inlineStr">
         <is>
           <t>Expirada</t>
         </is>
       </c>
-      <c r="J45" t="inlineStr">
+      <c r="K45" t="inlineStr">
         <is>
           <t>2025-11-13T15:27:36.746Z</t>
         </is>
       </c>
-      <c r="K45" t="inlineStr"/>
       <c r="L45" t="inlineStr"/>
       <c r="M45" t="inlineStr"/>
-      <c r="N45" t="inlineStr">
+      <c r="N45" t="inlineStr"/>
+      <c r="O45" t="inlineStr">
         <is>
           <t>Kaue Teixeira Caldeira Venâncio</t>
         </is>
       </c>
-      <c r="O45" t="inlineStr"/>
-      <c r="P45" t="inlineStr">
+      <c r="P45" t="inlineStr"/>
+      <c r="Q45" t="inlineStr">
         <is>
           <t>2025-11-06T15:27:46.917Z</t>
         </is>
       </c>
-      <c r="Q45" t="inlineStr">
+      <c r="R45" t="inlineStr">
         <is>
           <t>NzdmMmMwZTItZWIyMy00ODUzLWJiZTgtM2Y3YTgzNGM0YzRmOjU3MDE2</t>
         </is>
       </c>
-      <c r="R45" t="inlineStr">
+      <c r="S45" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="S45" t="inlineStr">
+      <c r="T45" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="T45" t="inlineStr">
+      <c r="U45" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U45" t="inlineStr">
+      <c r="V45" t="inlineStr">
         <is>
           <t>MzU0MDM4MDo1NzAxNg==</t>
         </is>
       </c>
-      <c r="V45" t="inlineStr">
+      <c r="W45" t="inlineStr">
         <is>
           <t>MzNhMjk0ZTUtMzI4MS00YTMwLTg2Y2QtYzM3YTQ0OTAyNzI5OjU3MDE2</t>
         </is>
       </c>
-      <c r="W45" t="inlineStr">
+      <c r="X45" t="inlineStr">
         <is>
           <t>expired</t>
         </is>
@@ -4803,57 +4852,58 @@
           <t>428</t>
         </is>
       </c>
-      <c r="I46" t="inlineStr">
+      <c r="I46" t="inlineStr"/>
+      <c r="J46" t="inlineStr">
         <is>
           <t>Expirada</t>
         </is>
       </c>
-      <c r="J46" t="inlineStr">
+      <c r="K46" t="inlineStr">
         <is>
           <t>2026-02-02T19:59:46.198Z</t>
         </is>
       </c>
-      <c r="K46" t="inlineStr"/>
       <c r="L46" t="inlineStr"/>
       <c r="M46" t="inlineStr"/>
-      <c r="N46" t="inlineStr">
+      <c r="N46" t="inlineStr"/>
+      <c r="O46" t="inlineStr">
         <is>
           <t>Lucas Uenishi Tada</t>
         </is>
       </c>
-      <c r="O46" t="inlineStr"/>
-      <c r="P46" t="inlineStr">
+      <c r="P46" t="inlineStr"/>
+      <c r="Q46" t="inlineStr">
         <is>
           <t>2026-01-26T20:04:54.521Z</t>
         </is>
       </c>
-      <c r="Q46" t="inlineStr"/>
-      <c r="R46" t="inlineStr">
+      <c r="R46" t="inlineStr"/>
+      <c r="S46" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="S46" t="inlineStr">
+      <c r="T46" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="T46" t="inlineStr">
+      <c r="U46" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U46" t="inlineStr">
+      <c r="V46" t="inlineStr">
         <is>
           <t>MzQwMzM1ODo1NzAxNg==</t>
         </is>
       </c>
-      <c r="V46" t="inlineStr">
+      <c r="W46" t="inlineStr">
         <is>
           <t>ZjUzOGNhMTktYmI4Yi00MmUwLTk4ZDYtYzQyNzk3M2U2ZWE2OjU3MDE2</t>
         </is>
       </c>
-      <c r="W46" t="inlineStr">
+      <c r="X46" t="inlineStr">
         <is>
           <t>expired</t>
         </is>
@@ -4894,57 +4944,58 @@
           <t>2123.15</t>
         </is>
       </c>
-      <c r="I47" t="inlineStr">
+      <c r="I47" t="inlineStr"/>
+      <c r="J47" t="inlineStr">
         <is>
           <t>Expirada</t>
         </is>
       </c>
-      <c r="J47" t="inlineStr">
+      <c r="K47" t="inlineStr">
         <is>
           <t>2025-11-04T13:33:37.491Z</t>
         </is>
       </c>
-      <c r="K47" t="inlineStr"/>
       <c r="L47" t="inlineStr"/>
       <c r="M47" t="inlineStr"/>
-      <c r="N47" t="inlineStr">
+      <c r="N47" t="inlineStr"/>
+      <c r="O47" t="inlineStr">
         <is>
           <t>Kaue Teixeira Caldeira Venâncio</t>
         </is>
       </c>
-      <c r="O47" t="inlineStr"/>
-      <c r="P47" t="inlineStr">
+      <c r="P47" t="inlineStr"/>
+      <c r="Q47" t="inlineStr">
         <is>
           <t>2025-10-28T14:06:21.222Z</t>
         </is>
       </c>
-      <c r="Q47" t="inlineStr"/>
-      <c r="R47" t="inlineStr">
+      <c r="R47" t="inlineStr"/>
+      <c r="S47" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="S47" t="inlineStr">
+      <c r="T47" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="T47" t="inlineStr">
+      <c r="U47" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U47" t="inlineStr">
+      <c r="V47" t="inlineStr">
         <is>
           <t>NDgyMTM3Mjo1NzAxNg==</t>
         </is>
       </c>
-      <c r="V47" t="inlineStr">
+      <c r="W47" t="inlineStr">
         <is>
           <t>MjIwOTU3OGEtZGZlNi00Njk1LThhZWQtNjM5YzVjZjJmZTg5OjU3MDE2</t>
         </is>
       </c>
-      <c r="W47" t="inlineStr">
+      <c r="X47" t="inlineStr">
         <is>
           <t>expired</t>
         </is>
@@ -4985,65 +5036,66 @@
           <t>511.65999999999997</t>
         </is>
       </c>
-      <c r="I48" t="inlineStr">
+      <c r="I48" t="inlineStr"/>
+      <c r="J48" t="inlineStr">
         <is>
           <t>Aprovada</t>
         </is>
       </c>
-      <c r="J48" t="inlineStr">
+      <c r="K48" t="inlineStr">
         <is>
           <t>2025-11-10T14:43:09.194Z</t>
         </is>
       </c>
-      <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr"/>
-      <c r="M48" t="inlineStr">
+      <c r="M48" t="inlineStr"/>
+      <c r="N48" t="inlineStr">
         <is>
           <t>Viktor Chagas</t>
         </is>
       </c>
-      <c r="N48" t="inlineStr">
+      <c r="O48" t="inlineStr">
         <is>
           <t>Kaue Teixeira Caldeira Venâncio</t>
         </is>
       </c>
-      <c r="O48" t="inlineStr">
+      <c r="P48" t="inlineStr">
         <is>
           <t>accounts/57016/quotations/cd11dd30-d3a2-4b5d-86e1-b7227ae83528/signatures/a288c6fe-a015-4ab6-8ff4-5716e239b3f1.png</t>
         </is>
       </c>
-      <c r="P48" t="inlineStr">
+      <c r="Q48" t="inlineStr">
         <is>
           <t>2025-11-03T15:08:36.141Z</t>
         </is>
       </c>
-      <c r="Q48" t="inlineStr"/>
-      <c r="R48" t="inlineStr">
+      <c r="R48" t="inlineStr"/>
+      <c r="S48" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="S48" t="inlineStr">
+      <c r="T48" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="T48" t="inlineStr">
+      <c r="U48" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U48" t="inlineStr">
+      <c r="V48" t="inlineStr">
         <is>
           <t>MzkzMzA3Mjo1NzAxNg==</t>
         </is>
       </c>
-      <c r="V48" t="inlineStr">
+      <c r="W48" t="inlineStr">
         <is>
           <t>ZmU3NjFlZTktOWMxMy00OWM5LTlkZWItZjU0NGMzZjM3YTBkOjU3MDE2</t>
         </is>
       </c>
-      <c r="W48" t="inlineStr">
+      <c r="X48" t="inlineStr">
         <is>
           <t>approved</t>
         </is>
@@ -5084,65 +5136,66 @@
           <t>552</t>
         </is>
       </c>
-      <c r="I49" t="inlineStr">
+      <c r="I49" t="inlineStr"/>
+      <c r="J49" t="inlineStr">
         <is>
           <t>Cancelada</t>
         </is>
       </c>
-      <c r="J49" t="inlineStr">
+      <c r="K49" t="inlineStr">
         <is>
           <t>2026-02-02T19:52:49.086Z</t>
         </is>
       </c>
-      <c r="K49" t="inlineStr">
+      <c r="L49" t="inlineStr">
         <is>
           <t>2026-01-27T12:28:33.000Z</t>
         </is>
       </c>
-      <c r="L49" t="inlineStr">
+      <c r="M49" t="inlineStr">
         <is>
           <t>2026-01-27T12:28:33.000Z</t>
         </is>
       </c>
-      <c r="M49" t="inlineStr"/>
-      <c r="N49" t="inlineStr">
+      <c r="N49" t="inlineStr"/>
+      <c r="O49" t="inlineStr">
         <is>
           <t>Lucas Uenishi Tada</t>
         </is>
       </c>
-      <c r="O49" t="inlineStr"/>
-      <c r="P49" t="inlineStr">
+      <c r="P49" t="inlineStr"/>
+      <c r="Q49" t="inlineStr">
         <is>
           <t>2026-01-26T19:59:17.023Z</t>
         </is>
       </c>
-      <c r="Q49" t="inlineStr"/>
-      <c r="R49" t="inlineStr">
+      <c r="R49" t="inlineStr"/>
+      <c r="S49" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="S49" t="inlineStr">
+      <c r="T49" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="T49" t="inlineStr">
+      <c r="U49" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U49" t="inlineStr">
+      <c r="V49" t="inlineStr">
         <is>
           <t>MzM3ODQxNDo1NzAxNg==</t>
         </is>
       </c>
-      <c r="V49" t="inlineStr">
+      <c r="W49" t="inlineStr">
         <is>
           <t>MTZkNGJlZmQtNjNlNC00MWQ1LWEzNTEtODYxOWM3N2JmMzQ3OjU3MDE2</t>
         </is>
       </c>
-      <c r="W49" t="inlineStr">
+      <c r="X49" t="inlineStr">
         <is>
           <t>canceled</t>
         </is>
@@ -5185,61 +5238,62 @@
           <t>350</t>
         </is>
       </c>
-      <c r="I50" t="inlineStr">
+      <c r="I50" t="inlineStr"/>
+      <c r="J50" t="inlineStr">
         <is>
           <t>Expirada</t>
         </is>
       </c>
-      <c r="J50" t="inlineStr">
+      <c r="K50" t="inlineStr">
         <is>
           <t>2025-12-09T18:46:05.954Z</t>
         </is>
       </c>
-      <c r="K50" t="inlineStr"/>
       <c r="L50" t="inlineStr"/>
       <c r="M50" t="inlineStr"/>
-      <c r="N50" t="inlineStr">
+      <c r="N50" t="inlineStr"/>
+      <c r="O50" t="inlineStr">
         <is>
           <t>Adriana Vieira Masini</t>
         </is>
       </c>
-      <c r="O50" t="inlineStr"/>
-      <c r="P50" t="inlineStr">
+      <c r="P50" t="inlineStr"/>
+      <c r="Q50" t="inlineStr">
         <is>
           <t>2025-12-02T18:53:10.136Z</t>
         </is>
       </c>
-      <c r="Q50" t="inlineStr">
+      <c r="R50" t="inlineStr">
         <is>
           <t>ODAxNDQ5MTMtNDYwMi00MjhmLWE1MWUtMWY1Y2I5NGIxY2Y1OjU3MDE2</t>
         </is>
       </c>
-      <c r="R50" t="inlineStr">
+      <c r="S50" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="S50" t="inlineStr">
+      <c r="T50" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="T50" t="inlineStr">
+      <c r="U50" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U50" t="inlineStr">
+      <c r="V50" t="inlineStr">
         <is>
           <t>MzMzMDQ1Mjo1NzAxNg==</t>
         </is>
       </c>
-      <c r="V50" t="inlineStr">
+      <c r="W50" t="inlineStr">
         <is>
           <t>ZTU1NzI4MzEtZTkzNS00ZWIzLTk4MTktMGE3MTZhOTE1NDZlOjU3MDE2</t>
         </is>
       </c>
-      <c r="W50" t="inlineStr">
+      <c r="X50" t="inlineStr">
         <is>
           <t>expired</t>
         </is>
@@ -5280,61 +5334,62 @@
           <t>979.73</t>
         </is>
       </c>
-      <c r="I51" t="inlineStr">
+      <c r="I51" t="inlineStr"/>
+      <c r="J51" t="inlineStr">
         <is>
           <t>Expirada</t>
         </is>
       </c>
-      <c r="J51" t="inlineStr">
+      <c r="K51" t="inlineStr">
         <is>
           <t>2025-11-13T15:27:16.361Z</t>
         </is>
       </c>
-      <c r="K51" t="inlineStr"/>
       <c r="L51" t="inlineStr"/>
       <c r="M51" t="inlineStr"/>
-      <c r="N51" t="inlineStr">
+      <c r="N51" t="inlineStr"/>
+      <c r="O51" t="inlineStr">
         <is>
           <t>Kaue Teixeira Caldeira Venâncio</t>
         </is>
       </c>
-      <c r="O51" t="inlineStr"/>
-      <c r="P51" t="inlineStr">
+      <c r="P51" t="inlineStr"/>
+      <c r="Q51" t="inlineStr">
         <is>
           <t>2025-11-06T15:27:31.134Z</t>
         </is>
       </c>
-      <c r="Q51" t="inlineStr">
+      <c r="R51" t="inlineStr">
         <is>
           <t>NzdmMmMwZTItZWIyMy00ODUzLWJiZTgtM2Y3YTgzNGM0YzRmOjU3MDE2</t>
         </is>
       </c>
-      <c r="R51" t="inlineStr">
+      <c r="S51" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="S51" t="inlineStr">
+      <c r="T51" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="T51" t="inlineStr">
+      <c r="U51" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U51" t="inlineStr">
+      <c r="V51" t="inlineStr">
         <is>
           <t>MzU0MDM4MDo1NzAxNg==</t>
         </is>
       </c>
-      <c r="V51" t="inlineStr">
+      <c r="W51" t="inlineStr">
         <is>
           <t>MzNhMjk0ZTUtMzI4MS00YTMwLTg2Y2QtYzM3YTQ0OTAyNzI5OjU3MDE2</t>
         </is>
       </c>
-      <c r="W51" t="inlineStr">
+      <c r="X51" t="inlineStr">
         <is>
           <t>expired</t>
         </is>
@@ -5375,61 +5430,62 @@
           <t>1224.475</t>
         </is>
       </c>
-      <c r="I52" t="inlineStr">
+      <c r="I52" t="inlineStr"/>
+      <c r="J52" t="inlineStr">
         <is>
           <t>Expirada</t>
         </is>
       </c>
-      <c r="J52" t="inlineStr">
+      <c r="K52" t="inlineStr">
         <is>
           <t>2026-01-02T18:34:01.969Z</t>
         </is>
       </c>
-      <c r="K52" t="inlineStr"/>
       <c r="L52" t="inlineStr"/>
       <c r="M52" t="inlineStr"/>
-      <c r="N52" t="inlineStr">
+      <c r="N52" t="inlineStr"/>
+      <c r="O52" t="inlineStr">
         <is>
           <t>Adriana Vieira Masini</t>
         </is>
       </c>
-      <c r="O52" t="inlineStr"/>
-      <c r="P52" t="inlineStr">
+      <c r="P52" t="inlineStr"/>
+      <c r="Q52" t="inlineStr">
         <is>
           <t>2025-12-26T18:48:40.881Z</t>
         </is>
       </c>
-      <c r="Q52" t="inlineStr">
+      <c r="R52" t="inlineStr">
         <is>
           <t>ODAxNDQ5MTMtNDYwMi00MjhmLWE1MWUtMWY1Y2I5NGIxY2Y1OjU3MDE2</t>
         </is>
       </c>
-      <c r="R52" t="inlineStr">
+      <c r="S52" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="S52" t="inlineStr">
+      <c r="T52" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="T52" t="inlineStr">
+      <c r="U52" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U52" t="inlineStr">
+      <c r="V52" t="inlineStr">
         <is>
           <t>MzMzMDQ1Mjo1NzAxNg==</t>
         </is>
       </c>
-      <c r="V52" t="inlineStr">
+      <c r="W52" t="inlineStr">
         <is>
           <t>ZTU1NzI4MzEtZTkzNS00ZWIzLTk4MTktMGE3MTZhOTE1NDZlOjU3MDE2</t>
         </is>
       </c>
-      <c r="W52" t="inlineStr">
+      <c r="X52" t="inlineStr">
         <is>
           <t>expired</t>
         </is>
@@ -5466,61 +5522,62 @@
           <t>1172.55</t>
         </is>
       </c>
-      <c r="I53" t="inlineStr">
+      <c r="I53" t="inlineStr"/>
+      <c r="J53" t="inlineStr">
         <is>
           <t>Expirada</t>
         </is>
       </c>
-      <c r="J53" t="inlineStr">
+      <c r="K53" t="inlineStr">
         <is>
           <t>2025-10-20T12:26:24.223Z</t>
         </is>
       </c>
-      <c r="K53" t="inlineStr"/>
       <c r="L53" t="inlineStr"/>
       <c r="M53" t="inlineStr"/>
-      <c r="N53" t="inlineStr">
+      <c r="N53" t="inlineStr"/>
+      <c r="O53" t="inlineStr">
         <is>
           <t>Adriana Vieira Masini</t>
         </is>
       </c>
-      <c r="O53" t="inlineStr"/>
-      <c r="P53" t="inlineStr">
+      <c r="P53" t="inlineStr"/>
+      <c r="Q53" t="inlineStr">
         <is>
           <t>2025-10-13T12:45:43.188Z</t>
         </is>
       </c>
-      <c r="Q53" t="inlineStr">
+      <c r="R53" t="inlineStr">
         <is>
           <t>MjkyMTJlNzYtODY0OC00NTBhLTg0OTUtOThlZGQ5YzM1MDdiOjU3MDE2</t>
         </is>
       </c>
-      <c r="R53" t="inlineStr">
+      <c r="S53" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="S53" t="inlineStr">
+      <c r="T53" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="T53" t="inlineStr">
+      <c r="U53" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U53" t="inlineStr">
+      <c r="V53" t="inlineStr">
         <is>
           <t>MzQ2NDM2Nzo1NzAxNg==</t>
         </is>
       </c>
-      <c r="V53" t="inlineStr">
+      <c r="W53" t="inlineStr">
         <is>
           <t>ZjQzMjRhOTEtZWM2NC00ZWUzLWFmNWItODM5NDliOWM2MjkzOjU3MDE2</t>
         </is>
       </c>
-      <c r="W53" t="inlineStr">
+      <c r="X53" t="inlineStr">
         <is>
           <t>expired</t>
         </is>
@@ -5561,65 +5618,66 @@
           <t>850.76</t>
         </is>
       </c>
-      <c r="I54" t="inlineStr">
+      <c r="I54" t="inlineStr"/>
+      <c r="J54" t="inlineStr">
         <is>
           <t>Cancelada</t>
         </is>
       </c>
-      <c r="J54" t="inlineStr">
+      <c r="K54" t="inlineStr">
         <is>
           <t>2026-01-27T19:00:18.732Z</t>
         </is>
       </c>
-      <c r="K54" t="inlineStr">
+      <c r="L54" t="inlineStr">
         <is>
           <t>2026-01-20T19:19:25.000Z</t>
         </is>
       </c>
-      <c r="L54" t="inlineStr">
+      <c r="M54" t="inlineStr">
         <is>
           <t>2026-01-20T19:19:25.000Z</t>
         </is>
       </c>
-      <c r="M54" t="inlineStr"/>
-      <c r="N54" t="inlineStr">
+      <c r="N54" t="inlineStr"/>
+      <c r="O54" t="inlineStr">
         <is>
           <t>Lucas Uenishi Tada</t>
         </is>
       </c>
-      <c r="O54" t="inlineStr"/>
-      <c r="P54" t="inlineStr">
+      <c r="P54" t="inlineStr"/>
+      <c r="Q54" t="inlineStr">
         <is>
           <t>2026-01-20T19:17:25.784Z</t>
         </is>
       </c>
-      <c r="Q54" t="inlineStr"/>
-      <c r="R54" t="inlineStr">
+      <c r="R54" t="inlineStr"/>
+      <c r="S54" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="S54" t="inlineStr">
+      <c r="T54" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="T54" t="inlineStr">
+      <c r="U54" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U54" t="inlineStr">
+      <c r="V54" t="inlineStr">
         <is>
           <t>NDM1ODE3Nzo1NzAxNg==</t>
         </is>
       </c>
-      <c r="V54" t="inlineStr">
+      <c r="W54" t="inlineStr">
         <is>
           <t>ZDBlYTE4ZjgtNTRlNS00YjQ2LWIwZDEtZmM2MDc4ZTFhYjY1OjU3MDE2</t>
         </is>
       </c>
-      <c r="W54" t="inlineStr">
+      <c r="X54" t="inlineStr">
         <is>
           <t>canceled</t>
         </is>
@@ -5660,61 +5718,62 @@
           <t>683</t>
         </is>
       </c>
-      <c r="I55" t="inlineStr">
+      <c r="I55" t="inlineStr"/>
+      <c r="J55" t="inlineStr">
         <is>
           <t>Expirada</t>
         </is>
       </c>
-      <c r="J55" t="inlineStr">
+      <c r="K55" t="inlineStr">
         <is>
           <t>2026-01-21T15:16:56.016Z</t>
         </is>
       </c>
-      <c r="K55" t="inlineStr"/>
       <c r="L55" t="inlineStr"/>
       <c r="M55" t="inlineStr"/>
-      <c r="N55" t="inlineStr">
+      <c r="N55" t="inlineStr"/>
+      <c r="O55" t="inlineStr">
         <is>
           <t>Adriana Vieira Masini</t>
         </is>
       </c>
-      <c r="O55" t="inlineStr"/>
-      <c r="P55" t="inlineStr">
+      <c r="P55" t="inlineStr"/>
+      <c r="Q55" t="inlineStr">
         <is>
           <t>2026-01-14T15:28:26.334Z</t>
         </is>
       </c>
-      <c r="Q55" t="inlineStr">
+      <c r="R55" t="inlineStr">
         <is>
           <t>NmQyZWFkMDctOWI5NC00YjQxLTgyZjYtN2VjYTAyYzM5ZTFiOjU3MDE2</t>
         </is>
       </c>
-      <c r="R55" t="inlineStr">
+      <c r="S55" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="S55" t="inlineStr">
+      <c r="T55" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="T55" t="inlineStr">
+      <c r="U55" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U55" t="inlineStr">
+      <c r="V55" t="inlineStr">
         <is>
           <t>NDgzNTU3MTo1NzAxNg==</t>
         </is>
       </c>
-      <c r="V55" t="inlineStr">
+      <c r="W55" t="inlineStr">
         <is>
           <t>Zjk2NjZmMDUtZjI0Ny00MTQxLWJmMmItMzZhOWRkNzNlYzgwOjU3MDE2</t>
         </is>
       </c>
-      <c r="W55" t="inlineStr">
+      <c r="X55" t="inlineStr">
         <is>
           <t>expired</t>
         </is>
@@ -5759,61 +5818,62 @@
           <t>1047.65</t>
         </is>
       </c>
-      <c r="I56" t="inlineStr">
+      <c r="I56" t="inlineStr"/>
+      <c r="J56" t="inlineStr">
         <is>
           <t>Expirada</t>
         </is>
       </c>
-      <c r="J56" t="inlineStr">
+      <c r="K56" t="inlineStr">
         <is>
           <t>2025-10-14T18:12:15.015Z</t>
         </is>
       </c>
-      <c r="K56" t="inlineStr"/>
       <c r="L56" t="inlineStr"/>
       <c r="M56" t="inlineStr"/>
-      <c r="N56" t="inlineStr">
+      <c r="N56" t="inlineStr"/>
+      <c r="O56" t="inlineStr">
         <is>
           <t>Adriana Vieira Masini</t>
         </is>
       </c>
-      <c r="O56" t="inlineStr"/>
-      <c r="P56" t="inlineStr">
+      <c r="P56" t="inlineStr"/>
+      <c r="Q56" t="inlineStr">
         <is>
           <t>2025-10-07T18:22:28.553Z</t>
         </is>
       </c>
-      <c r="Q56" t="inlineStr">
+      <c r="R56" t="inlineStr">
         <is>
           <t>ODZlODFiMWItM2FiOC00YmY2LWJiOTktMTExOWE5YzVjMDBjOjU3MDE2</t>
         </is>
       </c>
-      <c r="R56" t="inlineStr">
+      <c r="S56" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="S56" t="inlineStr">
+      <c r="T56" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="T56" t="inlineStr">
+      <c r="U56" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U56" t="inlineStr">
+      <c r="V56" t="inlineStr">
         <is>
           <t>MzI2OTMyNjo1NzAxNg==</t>
         </is>
       </c>
-      <c r="V56" t="inlineStr">
+      <c r="W56" t="inlineStr">
         <is>
           <t>MWUzYmI1OWItNmZiNC00ODg1LTg0ODktOTlmY2IyZWYxNWIxOjU3MDE2</t>
         </is>
       </c>
-      <c r="W56" t="inlineStr">
+      <c r="X56" t="inlineStr">
         <is>
           <t>expired</t>
         </is>
@@ -5850,65 +5910,66 @@
           <t>40.894999999999996</t>
         </is>
       </c>
-      <c r="I57" t="inlineStr">
+      <c r="I57" t="inlineStr"/>
+      <c r="J57" t="inlineStr">
         <is>
           <t>Aprovada</t>
         </is>
       </c>
-      <c r="J57" t="inlineStr">
+      <c r="K57" t="inlineStr">
         <is>
           <t>2025-11-11T15:57:22.457Z</t>
         </is>
       </c>
-      <c r="K57" t="inlineStr"/>
       <c r="L57" t="inlineStr"/>
-      <c r="M57" t="inlineStr">
+      <c r="M57" t="inlineStr"/>
+      <c r="N57" t="inlineStr">
         <is>
           <t>Marcos</t>
         </is>
       </c>
-      <c r="N57" t="inlineStr">
+      <c r="O57" t="inlineStr">
         <is>
           <t>Kaue Teixeira Caldeira Venâncio</t>
         </is>
       </c>
-      <c r="O57" t="inlineStr">
+      <c r="P57" t="inlineStr">
         <is>
           <t>accounts/57016/quotations/e9de7ba0-386a-464d-8581-a8798001ad78/signatures/a05c1641-9b6c-465a-90ae-a4510b4e3986.png</t>
         </is>
       </c>
-      <c r="P57" t="inlineStr">
+      <c r="Q57" t="inlineStr">
         <is>
           <t>2025-11-04T15:57:50.841Z</t>
         </is>
       </c>
-      <c r="Q57" t="inlineStr"/>
-      <c r="R57" t="inlineStr">
+      <c r="R57" t="inlineStr"/>
+      <c r="S57" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="S57" t="inlineStr">
+      <c r="T57" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="T57" t="inlineStr">
+      <c r="U57" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U57" t="inlineStr">
+      <c r="V57" t="inlineStr">
         <is>
           <t>NDgyNTIyNjo1NzAxNg==</t>
         </is>
       </c>
-      <c r="V57" t="inlineStr">
+      <c r="W57" t="inlineStr">
         <is>
           <t>YTg2MWYxNTktMTEyNi00YWYxLWI4MmMtNzBlODk1NDQwMjE3OjU3MDE2</t>
         </is>
       </c>
-      <c r="W57" t="inlineStr">
+      <c r="X57" t="inlineStr">
         <is>
           <t>approved</t>
         </is>
@@ -5950,61 +6011,62 @@
           <t>549.22</t>
         </is>
       </c>
-      <c r="I58" t="inlineStr">
+      <c r="I58" t="inlineStr"/>
+      <c r="J58" t="inlineStr">
         <is>
           <t>Expirada</t>
         </is>
       </c>
-      <c r="J58" t="inlineStr">
+      <c r="K58" t="inlineStr">
         <is>
           <t>2025-10-06T19:05:55.326Z</t>
         </is>
       </c>
-      <c r="K58" t="inlineStr"/>
       <c r="L58" t="inlineStr"/>
       <c r="M58" t="inlineStr"/>
-      <c r="N58" t="inlineStr">
+      <c r="N58" t="inlineStr"/>
+      <c r="O58" t="inlineStr">
         <is>
           <t>Adriana Vieira Masini</t>
         </is>
       </c>
-      <c r="O58" t="inlineStr"/>
-      <c r="P58" t="inlineStr">
+      <c r="P58" t="inlineStr"/>
+      <c r="Q58" t="inlineStr">
         <is>
           <t>2025-09-29T20:26:53.403Z</t>
         </is>
       </c>
-      <c r="Q58" t="inlineStr">
+      <c r="R58" t="inlineStr">
         <is>
           <t>MDBmZTJkNzktN2M1YS00MDc0LWE2YTctNzZiZGNkZWFmYTIwOjU3MDE2</t>
         </is>
       </c>
-      <c r="R58" t="inlineStr">
+      <c r="S58" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="S58" t="inlineStr">
+      <c r="T58" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="T58" t="inlineStr">
+      <c r="U58" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U58" t="inlineStr">
+      <c r="V58" t="inlineStr">
         <is>
           <t>NDgyNTE1Mzo1NzAxNg==</t>
         </is>
       </c>
-      <c r="V58" t="inlineStr">
+      <c r="W58" t="inlineStr">
         <is>
           <t>MTcwZjFjYjQtMmE0OC00ZTYyLTg4ODAtZjBlOGU3M2I1MmExOjU3MDE2</t>
         </is>
       </c>
-      <c r="W58" t="inlineStr">
+      <c r="X58" t="inlineStr">
         <is>
           <t>expired</t>
         </is>
@@ -6045,61 +6107,62 @@
           <t>7000</t>
         </is>
       </c>
-      <c r="I59" t="inlineStr">
+      <c r="I59" t="inlineStr"/>
+      <c r="J59" t="inlineStr">
         <is>
           <t>Expirada</t>
         </is>
       </c>
-      <c r="J59" t="inlineStr">
+      <c r="K59" t="inlineStr">
         <is>
           <t>2026-02-06T18:27:35.984Z</t>
         </is>
       </c>
-      <c r="K59" t="inlineStr"/>
       <c r="L59" t="inlineStr"/>
       <c r="M59" t="inlineStr"/>
-      <c r="N59" t="inlineStr">
+      <c r="N59" t="inlineStr"/>
+      <c r="O59" t="inlineStr">
         <is>
           <t>Adriana Vieira Masini</t>
         </is>
       </c>
-      <c r="O59" t="inlineStr"/>
-      <c r="P59" t="inlineStr">
+      <c r="P59" t="inlineStr"/>
+      <c r="Q59" t="inlineStr">
         <is>
           <t>2026-01-30T18:40:19.770Z</t>
         </is>
       </c>
-      <c r="Q59" t="inlineStr">
+      <c r="R59" t="inlineStr">
         <is>
           <t>MDU1N2Q3Y2ItZmMxYi00OGVhLThkNDUtNzE5OGI0YjUwMWJkOjU3MDE2</t>
         </is>
       </c>
-      <c r="R59" t="inlineStr">
+      <c r="S59" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="S59" t="inlineStr">
+      <c r="T59" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="T59" t="inlineStr">
+      <c r="U59" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U59" t="inlineStr">
+      <c r="V59" t="inlineStr">
         <is>
           <t>NDM1ODE5OTo1NzAxNg==</t>
         </is>
       </c>
-      <c r="V59" t="inlineStr">
+      <c r="W59" t="inlineStr">
         <is>
           <t>NzYwMWZlNDAtMzg2Mi00YjcyLTgwYWEtYzdkNWM1YmZiYmZjOjU3MDE2</t>
         </is>
       </c>
-      <c r="W59" t="inlineStr">
+      <c r="X59" t="inlineStr">
         <is>
           <t>expired</t>
         </is>
@@ -6140,57 +6203,58 @@
           <t>2123.15</t>
         </is>
       </c>
-      <c r="I60" t="inlineStr">
+      <c r="I60" t="inlineStr"/>
+      <c r="J60" t="inlineStr">
         <is>
           <t>Expirada</t>
         </is>
       </c>
-      <c r="J60" t="inlineStr">
+      <c r="K60" t="inlineStr">
         <is>
           <t>2025-11-18T12:23:08.942Z</t>
         </is>
       </c>
-      <c r="K60" t="inlineStr"/>
       <c r="L60" t="inlineStr"/>
       <c r="M60" t="inlineStr"/>
-      <c r="N60" t="inlineStr">
+      <c r="N60" t="inlineStr"/>
+      <c r="O60" t="inlineStr">
         <is>
           <t>Kaue Teixeira Caldeira Venâncio</t>
         </is>
       </c>
-      <c r="O60" t="inlineStr"/>
-      <c r="P60" t="inlineStr">
+      <c r="P60" t="inlineStr"/>
+      <c r="Q60" t="inlineStr">
         <is>
           <t>2025-11-11T12:25:14.798Z</t>
         </is>
       </c>
-      <c r="Q60" t="inlineStr"/>
-      <c r="R60" t="inlineStr">
+      <c r="R60" t="inlineStr"/>
+      <c r="S60" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="S60" t="inlineStr">
+      <c r="T60" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="T60" t="inlineStr">
+      <c r="U60" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U60" t="inlineStr">
+      <c r="V60" t="inlineStr">
         <is>
           <t>NDgyMTM3Mjo1NzAxNg==</t>
         </is>
       </c>
-      <c r="V60" t="inlineStr">
+      <c r="W60" t="inlineStr">
         <is>
           <t>MjIwOTU3OGEtZGZlNi00Njk1LThhZWQtNjM5YzVjZjJmZTg5OjU3MDE2</t>
         </is>
       </c>
-      <c r="W60" t="inlineStr">
+      <c r="X60" t="inlineStr">
         <is>
           <t>expired</t>
         </is>
@@ -6227,69 +6291,70 @@
           <t>956.025</t>
         </is>
       </c>
-      <c r="I61" t="inlineStr">
+      <c r="I61" t="inlineStr"/>
+      <c r="J61" t="inlineStr">
         <is>
           <t>Aprovada</t>
         </is>
       </c>
-      <c r="J61" t="inlineStr">
+      <c r="K61" t="inlineStr">
         <is>
           <t>2025-11-21T18:23:47.104Z</t>
         </is>
       </c>
-      <c r="K61" t="inlineStr"/>
       <c r="L61" t="inlineStr"/>
-      <c r="M61" t="inlineStr">
+      <c r="M61" t="inlineStr"/>
+      <c r="N61" t="inlineStr">
         <is>
           <t>Débora Mendes Mangaba</t>
         </is>
       </c>
-      <c r="N61" t="inlineStr">
+      <c r="O61" t="inlineStr">
         <is>
           <t>Adriana Vieira Masini</t>
         </is>
       </c>
-      <c r="O61" t="inlineStr">
+      <c r="P61" t="inlineStr">
         <is>
           <t>accounts/57016/quotations/fbbec352-79e6-41e3-9553-a70ca4dd9b61/signatures/e629a18e-6cbe-4b79-8890-7071450b92a9.png</t>
         </is>
       </c>
-      <c r="P61" t="inlineStr">
+      <c r="Q61" t="inlineStr">
         <is>
           <t>2025-11-14T18:28:52.343Z</t>
         </is>
       </c>
-      <c r="Q61" t="inlineStr">
+      <c r="R61" t="inlineStr">
         <is>
           <t>ZWI1NTJkMzAtNjEwMS00NjM1LWE5MzYtOWE2ZTAwYjY2ZjgyOjU3MDE2</t>
         </is>
       </c>
-      <c r="R61" t="inlineStr">
+      <c r="S61" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="S61" t="inlineStr">
+      <c r="T61" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="T61" t="inlineStr">
+      <c r="U61" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U61" t="inlineStr">
+      <c r="V61" t="inlineStr">
         <is>
           <t>MzQwMzM1ODo1NzAxNg==</t>
         </is>
       </c>
-      <c r="V61" t="inlineStr">
+      <c r="W61" t="inlineStr">
         <is>
           <t>ZjUzOGNhMTktYmI4Yi00MmUwLTk4ZDYtYzQyNzk3M2U2ZWE2OjU3MDE2</t>
         </is>
       </c>
-      <c r="W61" t="inlineStr">
+      <c r="X61" t="inlineStr">
         <is>
           <t>approved</t>
         </is>
@@ -6330,61 +6395,62 @@
           <t>1197.8</t>
         </is>
       </c>
-      <c r="I62" t="inlineStr">
+      <c r="I62" t="inlineStr"/>
+      <c r="J62" t="inlineStr">
         <is>
           <t>Expirada</t>
         </is>
       </c>
-      <c r="J62" t="inlineStr">
+      <c r="K62" t="inlineStr">
         <is>
           <t>2026-01-02T18:19:58.819Z</t>
         </is>
       </c>
-      <c r="K62" t="inlineStr"/>
       <c r="L62" t="inlineStr"/>
       <c r="M62" t="inlineStr"/>
-      <c r="N62" t="inlineStr">
+      <c r="N62" t="inlineStr"/>
+      <c r="O62" t="inlineStr">
         <is>
           <t>Adriana Vieira Masini</t>
         </is>
       </c>
-      <c r="O62" t="inlineStr"/>
-      <c r="P62" t="inlineStr">
+      <c r="P62" t="inlineStr"/>
+      <c r="Q62" t="inlineStr">
         <is>
           <t>2025-12-26T18:30:18.349Z</t>
         </is>
       </c>
-      <c r="Q62" t="inlineStr">
+      <c r="R62" t="inlineStr">
         <is>
           <t>NDU4ZDY0OTgtYjQwNy00MTdhLWE5YjYtNTg5ZDcyNGExMTQ1OjU3MDE2</t>
         </is>
       </c>
-      <c r="R62" t="inlineStr">
+      <c r="S62" t="inlineStr">
         <is>
           <t>percentage</t>
         </is>
       </c>
-      <c r="S62" t="inlineStr">
+      <c r="T62" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="T62" t="inlineStr">
+      <c r="U62" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U62" t="inlineStr">
+      <c r="V62" t="inlineStr">
         <is>
           <t>NTE2MTc5NTo1NzAxNg==</t>
         </is>
       </c>
-      <c r="V62" t="inlineStr">
+      <c r="W62" t="inlineStr">
         <is>
           <t>ZTRkNTk4YzgtZTAxMi00ZWVkLWJkZTgtYTBkMjEzYmNkZjFiOjU3MDE2</t>
         </is>
       </c>
-      <c r="W62" t="inlineStr">
+      <c r="X62" t="inlineStr">
         <is>
           <t>expired</t>
         </is>

</xml_diff>